<commit_message>
ALITA v3.0.1 – first legal project: AI Act Commission proposal (REQ-41)
- _legal.yaml: file may be a list (main document + annexes = one version)
- Segmentation of Commission proposals: TITLE/CHAPTER levels, all annexes,
  numbered definitions, legislative financial statement as supplement,
  "EN n EN" footers, wrapped "Article 61." references, two-line headings
- Drafts-only fallback in the chats (latest draft, disclosed)
- Draft versions keep their own title ("AI Act – Proposal")
- Tests (81 passed), CHANGELOG, docs, requirements log

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiuZbjdoe5Dn8qVgxqM
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -553,10 +553,11 @@
     <row r="2" ht="15" customHeight="1" s="11">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>Stand: Release 3.0.0 vom 29.10.2026 · REQ-01 – REQ-21 aus dem Review von 2.0.0, REQ-22 – REQ-34 aus der Sitzung vom 17.10.2026 (inkl. Feedback von Dustin), REQ-35 – REQ-40 aus der Sitzung vom 29.10.2026</t>
-        </is>
-      </c>
-    </row>
+          <t>Stand: Release 3.0.1 vom 29.10.2026 · REQ-01 – REQ-21 aus dem Review von 2.0.0, REQ-22 – REQ-34 aus der Sitzung vom 17.10.2026 (inkl. Feedback von Dustin), REQ-35 – REQ-41 aus der Sitzung vom 29.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="11">
       <c r="A4" s="14" t="inlineStr">
         <is>
@@ -660,11 +661,11 @@
     <row r="13" ht="15" customHeight="1" s="11">
       <c r="A13" s="17" t="inlineStr">
         <is>
-          <t>Neu in Release 3.0.0</t>
+          <t>Neu in Release 3.0.x</t>
         </is>
       </c>
       <c r="B13" s="18">
-        <f>COUNTIF(Requirements!D2:D200,"3.0.0*")</f>
+        <f>COUNTIF(Requirements!D2:D200,"3.0.*")</f>
         <v/>
       </c>
     </row>
@@ -700,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -1990,7 +1991,7 @@
         </is>
       </c>
     </row>
-    <row r="41">
+    <row r="41" s="11">
       <c r="A41" s="22" t="inlineStr">
         <is>
           <t>REQ-40</t>
@@ -2019,6 +2020,38 @@
       <c r="F41" s="22" t="inlineStr">
         <is>
           <t>Beantwortet: DoCO, DEO, Pattern Ontology (Constantin et al. 2016), FaBiO und CiTO (Peroni &amp; Shotton 2012), BIBO (D’Arcus &amp; Giasson 2009), seit 3.0.0 ELI. Korrigiert: fabio:Note gibt es nicht → fabio:Expression; C4O aus der Doku entfernt (nie verwendet).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" s="11">
+      <c r="A42" s="22" t="inlineStr">
+        <is>
+          <t>REQ-41</t>
+        </is>
+      </c>
+      <c r="B42" s="22" t="inlineStr">
+        <is>
+          <t>Erstes Legal project einlesen: Kommissionsvorschlag AI Act (Hauptdokument + Anhänge)</t>
+        </is>
+      </c>
+      <c r="C42" s="22" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
+        </is>
+      </c>
+      <c r="D42" s="22" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="E42" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 29.10.2026</t>
+        </is>
+      </c>
+      <c r="F42" s="22" t="inlineStr">
+        <is>
+          <t>Dateien in research/EUAIA/legal/EU-AI-Act/ abgelegt, _legal.yaml mit file: [Hauptdokument, Anhänge] als eine Fassung. Parser für Kommissionsvorschläge erweitert (TITLE/CHAPTER, alle 9 Anhänge, Begriffsbestimmungen, Finanzbogen als Anlage, Seitenfüße „EN n EN“, umbrochene Verweise). Offline mit den echten PDFs geprüft: 85 Artikel, 89 Erwägungsgründe, 9 Anhänge, 699 Bestandteile, 889 Text Units. Rückfall auf den jüngsten Entwurf, wenn kein Gesetz gilt. Das Einlesen selbst (Embedding, Qdrant, Neo4j) läuft per Docker auf dem Server – noch auszuführen.</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -3055,7 +3088,7 @@
         </is>
       </c>
     </row>
-    <row r="20">
+    <row r="20" s="11">
       <c r="A20" s="22" t="inlineStr">
         <is>
           <t>REQ-40</t>
@@ -3104,6 +3137,58 @@
       <c r="J20" s="22" t="inlineStr">
         <is>
           <t>Literaturangaben im Chat geliefert; fabio:Note → fabio:Expression, C4O-Zeile entfernt (3.0.0).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" s="11">
+      <c r="A21" s="22" t="inlineStr">
+        <is>
+          <t>REQ-41</t>
+        </is>
+      </c>
+      <c r="B21" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C21" s="22" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="D21" s="22" t="inlineStr">
+        <is>
+          <t>Hier ist das erste legal project. ich hänge dir 2 dateien die ein dokument darstellen. kann man das einmal ingesten?</t>
+        </is>
+      </c>
+      <c r="E21" s="22" t="inlineStr">
+        <is>
+          <t>Ein Legal project MUSS aus Fassungen bestehen können, deren Text auf mehrere Dateien verteilt ist (Hauptdokument + Anhänge); der Kommissionsvorschlag COM(2021) 206 MUSS korrekt in Titel, Kapitel, Artikel, Absätze, Punkte, Erwägungsgründe und Anhänge zerlegt werden; der Finanzbogen DARF NICHT als Teil eines Artikels gelten. Sind nur Entwürfe vorhanden, SOLL der Chat den jüngsten Entwurf verwenden und das offenlegen.</t>
+        </is>
+      </c>
+      <c r="F21" s="22" t="inlineStr">
+        <is>
+          <t>Nach „ingest legal“ erscheint „AI Act – Proposal“ als ein Dokument (125 Seiten, beide Dateien) im Legal project „EU-AI-Act“ der Datenbank „EU AI Act“; 85 Artikel, 89 Erwägungsgründe, 9 Anhänge; Frage „What does Article 5 of the proposal prohibit?“ liefert Art. 5 mit Hinweis „Proposal, not in force“.</t>
+        </is>
+      </c>
+      <c r="G21" s="22" t="inlineStr">
+        <is>
+          <t>Backend · Ingest · Daten</t>
+        </is>
+      </c>
+      <c r="H21" s="22" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="I21" s="22" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
+        </is>
+      </c>
+      <c r="J21" s="22" t="inlineStr">
+        <is>
+          <t>Code + Tests fertig (81 passed), Modell offline aus den echten PDFs gebaut. Ingest im Docker-Container steht aus (in der Arbeitsumgebung kein Docker). Später: verabschiedete Verordnung 2024/1689 und konsolidierte Fassung ergänzen, dann mit --force neu einlesen.</t>
         </is>
       </c>
     </row>
@@ -3131,7 +3216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="130" customWidth="1" style="10" min="1" max="1"/>
@@ -3186,6 +3271,13 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="24" t="inlineStr">
+        <is>
+          <t>Release 3.0.1 (29.10.2026, Patch): REQ-41 (erstes Legal project – Kommissionsvorschlag des AI Act mit Anhängen) vorbereitet und offline geprüft; Einlesen per Docker ausstehend. Release Notes: CHANGELOG.md, Abschnitt [3.0.1].</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
ALITA v3.0.2 – re-cluster only the ingested databases (REQ-42)
- maybe_recluster: only the databases of the ingested data, each on its
  own, with projects or project files as in their last run; ingest all
  clusters the touched databases once at the end
- Legal project is one clustering unit; a database with one work gets a cluster
- Knowledge map: project labels no longer run over papers
- REQ-41 done (AI Act proposal ingested), REQ-42; tests 83 passed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiuZbjdoe5Dn8qVgxqM
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -553,7 +553,7 @@
     <row r="2" ht="15" customHeight="1" s="11">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>Stand: Release 3.0.1 vom 29.10.2026 · REQ-01 – REQ-21 aus dem Review von 2.0.0, REQ-22 – REQ-34 aus der Sitzung vom 17.10.2026 (inkl. Feedback von Dustin), REQ-35 – REQ-41 aus der Sitzung vom 29.10.2026</t>
+          <t>Stand: Release 3.0.2 vom 29.10.2026 · REQ-01 – REQ-21 aus dem Review von 2.0.0, REQ-22 – REQ-34 aus der Sitzung vom 17.10.2026 (inkl. Feedback von Dustin), REQ-35 – REQ-42 aus der Sitzung vom 29.10.2026</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -2036,7 +2036,7 @@
       </c>
       <c r="C42" s="22" t="inlineStr">
         <is>
-          <t>In Arbeit</t>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="D42" s="22" t="inlineStr">
@@ -2051,7 +2051,39 @@
       </c>
       <c r="F42" s="22" t="inlineStr">
         <is>
-          <t>Dateien in research/EUAIA/legal/EU-AI-Act/ abgelegt, _legal.yaml mit file: [Hauptdokument, Anhänge] als eine Fassung. Parser für Kommissionsvorschläge erweitert (TITLE/CHAPTER, alle 9 Anhänge, Begriffsbestimmungen, Finanzbogen als Anlage, Seitenfüße „EN n EN“, umbrochene Verweise). Offline mit den echten PDFs geprüft: 85 Artikel, 89 Erwägungsgründe, 9 Anhänge, 699 Bestandteile, 889 Text Units. Rückfall auf den jüngsten Entwurf, wenn kein Gesetz gilt. Das Einlesen selbst (Embedding, Qdrant, Neo4j) läuft per Docker auf dem Server – noch auszuführen.</t>
+          <t>Dateien in research/EUAIA/legal/EU-AI-Act/ abgelegt, _legal.yaml mit file: [Hauptdokument, Anhänge] als eine Fassung. Parser für Kommissionsvorschläge erweitert (TITLE/CHAPTER, alle 9 Anhänge, Begriffsbestimmungen, Finanzbogen als Anlage, Seitenfüße „EN n EN“, umbrochene Verweise). Offline mit den echten PDFs geprüft: 85 Artikel, 89 Erwägungsgründe, 9 Anhänge, 699 Bestandteile, 889 Text Units. Rückfall auf den jüngsten Entwurf, wenn kein Gesetz gilt. Am 29.10.2026 per Docker eingelesen (mit -e OPENROUTER_API_KEY).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" s="11">
+      <c r="A43" s="22" t="inlineStr">
+        <is>
+          <t>REQ-42</t>
+        </is>
+      </c>
+      <c r="B43" s="22" t="inlineStr">
+        <is>
+          <t>Wissenskarte nach dem Einlesen korrekt: bestehende Cluster bleiben erhalten</t>
+        </is>
+      </c>
+      <c r="C43" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="D43" s="22" t="inlineStr">
+        <is>
+          <t>3.0.2</t>
+        </is>
+      </c>
+      <c r="E43" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 29.10.2026</t>
+        </is>
+      </c>
+      <c r="F43" s="22" t="inlineStr">
+        <is>
+          <t>Ursache: automatisches Neu-Clustern nach der Ingestion lief über alle Datenbanken gemeinsam (k=3: 2× CNN_DM, 1× alle 74 Forschungswerke + AI Act) und überschrieb die Cluster je Datenbank. Jetzt nur die eingelesenen Datenbanken, jede für sich, mit ihrer bisherigen Einheit (Projekte/Projektdateien); Legal project als eine Einheit; Datenbank mit einem Werk bekommt einen Cluster; Projektbeschriftung überdeckt keine Paper mehr. Cluster der bestehenden Datenbanken einmalig neu berechnen (ingest cluster --db …, ML mit --files).</t>
         </is>
       </c>
     </row>
@@ -2086,7 +2118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -3183,12 +3215,64 @@
       </c>
       <c r="I21" s="22" t="inlineStr">
         <is>
-          <t>In Arbeit</t>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="J21" s="22" t="inlineStr">
         <is>
-          <t>Code + Tests fertig (81 passed), Modell offline aus den echten PDFs gebaut. Ingest im Docker-Container steht aus (in der Arbeitsumgebung kein Docker). Später: verabschiedete Verordnung 2024/1689 und konsolidierte Fassung ergänzen, dann mit --force neu einlesen.</t>
+          <t>Code + Tests fertig (81 passed), Modell offline aus den echten PDFs gebaut. Ingest per Docker am 29.10.2026 erfolgreich (erster Versuch scheiterte am fehlenden OpenRouter-Key – Key per -e OPENROUTER_API_KEY mitgeben). Später: Verordnung 2024/1689 und konsolidierte Fassung ergänzen, dann mit --force neu einlesen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" s="11">
+      <c r="A22" s="22" t="inlineStr">
+        <is>
+          <t>REQ-42</t>
+        </is>
+      </c>
+      <c r="B22" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C22" s="22" t="inlineStr">
+        <is>
+          <t>3.0.2</t>
+        </is>
+      </c>
+      <c r="D22" s="22" t="inlineStr">
+        <is>
+          <t>das ist ingested aber warum sieht das so falsch aus: [Screenshot der Wissenskarte: EU-AI-Act und alle Jasmine-Paper an einem Cluster C3]</t>
+        </is>
+      </c>
+      <c r="E22" s="22" t="inlineStr">
+        <is>
+          <t>Das Einlesen neuer Daten DARF die Cluster anderer Datenbanken NICHT verändern; nach einer Ingestion MÜSSEN nur die betroffenen Datenbanken neu geclustert werden, mit derselben Einheit wie zuvor (Projekte bzw. Projektdateien). Ein Legal project MUSS genau eine Clustering-Einheit sein. Beschriftungen in der Wissenskarte DÜRFEN andere Knoten NICHT überdecken.</t>
+        </is>
+      </c>
+      <c r="F22" s="22" t="inlineStr">
+        <is>
+          <t>Nach „ingest legal“ für EUAIA bleiben die Cluster von AL, DL, JSW, LDK, ML und CNN_DM unverändert; EUAIA hat einen eigenen Cluster; Auswahl Jasmine + EU AI Act zeigt Jasmines eigene Cluster und den AI Act getrennt; Projektname „EU-AI-Act“ überlappt kein Paper.</t>
+        </is>
+      </c>
+      <c r="G22" s="22" t="inlineStr">
+        <is>
+          <t>Backend · Clustering · Frontend</t>
+        </is>
+      </c>
+      <c r="H22" s="22" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="I22" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="J22" s="22" t="inlineStr">
+        <is>
+          <t>maybe_recluster(opts, databases) je DB mit _uses_project_files; ingest_all sammelt betroffene DBs; select_units ohne Legal-project-Doppel; recompute ab 1 Einheit; Label-Platz in clusters.js. Tests 83 passed. Bestehende Cluster müssen einmalig je DB neu berechnet werden.</t>
         </is>
       </c>
     </row>
@@ -3216,7 +3300,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="130" customWidth="1" style="10" min="1" max="1"/>
@@ -3278,6 +3362,13 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="24" t="inlineStr">
+        <is>
+          <t>Release 3.0.2 (29.10.2026, Patch): REQ-41 erledigt (AI-Act-Vorschlag eingelesen); REQ-42 (Clustering nach dem Einlesen nur für die betroffenen Datenbanken) erledigt. Release Notes: CHANGELOG.md, Abschnitt [3.0.2].</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
ALITA v3.1.0 – partial versions and the committee stage (REQ-43)
- _legal.yaml: partial: true – merge_partial takes missing components
  unchanged from the previous version, aligns structure, reading order
- Drafting stage "committee" (Parliament committee amendments), planner words
- Parser: compromise-amendment blocks (CA 1-12), article numbers "54 a",
  "28(a)", recitals "(65a)", repeated identical recitals once
- Version comparison by letters and digits only (cmp_key)
- AI Act: IMCO/LIBE draft compromise amendments (9.5.2023) as version 2
- Tests 86 passed, CHANGELOG, docs, requirements log

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiuZbjdoe5Dn8qVgxqM
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -553,7 +553,7 @@
     <row r="2" ht="15" customHeight="1" s="11">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>Stand: Release 3.0.2 vom 29.10.2026 · REQ-01 – REQ-21 aus dem Review von 2.0.0, REQ-22 – REQ-34 aus der Sitzung vom 17.10.2026 (inkl. Feedback von Dustin), REQ-35 – REQ-42 aus der Sitzung vom 29.10.2026</t>
+          <t>Stand: Release 3.1.0 vom 29.10.2026 · REQ-01 – REQ-21 aus dem Review von 2.0.0, REQ-22 – REQ-34 aus der Sitzung vom 17.10.2026 (inkl. Feedback von Dustin), REQ-35 – REQ-43 aus der Sitzung vom 29.10.2026</t>
         </is>
       </c>
     </row>
@@ -661,11 +661,11 @@
     <row r="13" ht="15" customHeight="1" s="11">
       <c r="A13" s="17" t="inlineStr">
         <is>
-          <t>Neu in Release 3.0.x</t>
+          <t>Neu in Release 3.x</t>
         </is>
       </c>
       <c r="B13" s="18">
-        <f>COUNTIF(Requirements!D2:D200,"3.0.*")</f>
+        <f>COUNTIF(Requirements!D2:D200,"3.*")</f>
         <v/>
       </c>
     </row>
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -2084,6 +2084,38 @@
       <c r="F43" s="22" t="inlineStr">
         <is>
           <t>Ursache: automatisches Neu-Clustern nach der Ingestion lief über alle Datenbanken gemeinsam (k=3: 2× CNN_DM, 1× alle 74 Forschungswerke + AI Act) und überschrieb die Cluster je Datenbank. Jetzt nur die eingelesenen Datenbanken, jede für sich, mit ihrer bisherigen Einheit (Projekte/Projektdateien); Legal project als eine Einheit; Datenbank mit einem Werk bekommt einen Cluster; Projektbeschriftung überdeckt keine Paper mehr. Cluster der bestehenden Datenbanken einmalig neu berechnen (ingest cluster --db …, ML mit --files).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" s="11">
+      <c r="A44" s="22" t="inlineStr">
+        <is>
+          <t>REQ-43</t>
+        </is>
+      </c>
+      <c r="B44" s="22" t="inlineStr">
+        <is>
+          <t>Nächste Fassung des AI Act: Kompromissänderungen IMCO/LIBE (9.5.2023) als Teilfassung</t>
+        </is>
+      </c>
+      <c r="C44" s="22" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
+        </is>
+      </c>
+      <c r="D44" s="22" t="inlineStr">
+        <is>
+          <t>3.1.0</t>
+        </is>
+      </c>
+      <c r="E44" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 29.10.2026</t>
+        </is>
+      </c>
+      <c r="F44" s="22" t="inlineStr">
+        <is>
+          <t>Datei abgelegt, _legal.yaml: Fassung 2 von 4, Stufe „committee“, partial: true. Neu: Teilfassungen (merge_partial – fehlende Teile unverändert aus der Vorfassung, keine Streichungen), Stufe committee im Planer, Parser für Kompromissblöcke CA 1–12, Artikelnummern „54 a“/„28(a)“, Erwägungsgründe „(65a)“, Vergleich nur über Buchstaben/Ziffern (cmp_key). Offline geprüft: 104 Artikel (24 neu), 129 Erwägungsgründe, 0 gestrichen, kleinste Änderungen echt (250 000 → 750 000 EUR, user → deployer). Einlesen per Docker steht aus.</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2150,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -3273,6 +3305,58 @@
       <c r="J22" s="22" t="inlineStr">
         <is>
           <t>maybe_recluster(opts, databases) je DB mit _uses_project_files; ingest_all sammelt betroffene DBs; select_units ohne Legal-project-Doppel; recompute ab 1 Einheit; Label-Platz in clusters.js. Tests 83 passed. Bestehende Cluster müssen einmalig je DB neu berechnet werden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" s="11">
+      <c r="A23" s="22" t="inlineStr">
+        <is>
+          <t>REQ-43</t>
+        </is>
+      </c>
+      <c r="B23" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C23" s="22" t="inlineStr">
+        <is>
+          <t>3.1.0</t>
+        </is>
+      </c>
+      <c r="D23" s="22" t="inlineStr">
+        <is>
+          <t>jetzt kommt das nächste dokument oder eine version vom ai act [ConsolidatedCA_IMCOLIBE_AI_ACT_EN.pdf]</t>
+        </is>
+      </c>
+      <c r="E23" s="22" t="inlineStr">
+        <is>
+          <t>Das Legal project „EU-AI-Act“ MUSS die Kompromissänderungen der Ausschüsse IMCO/LIBE vom 9.5.2023 als eigene Fassung (Entwurfsstufe, ohne Geltung) zwischen Vorschlag und Verordnung führen. Teile, die im Dokument nicht vorkommen, DÜRFEN NICHT als gestrichen gelten, sondern MÜSSEN aus der Vorfassung übernommen werden. Unterschiede der PDF-Extraktion (Leerzeichen, Bindestriche) DÜRFEN NICHT als Änderung zählen.</t>
+        </is>
+      </c>
+      <c r="F23" s="22" t="inlineStr">
+        <is>
+          <t>Nach „ingest legal“: zwei Fassungen (Proposal, Committee amendments); Fassung 2 mit 0 gestrichenen Bestandteilen; Art. 13 unverändert aus dem Vorschlag; neue Artikel 4a, 28a, 28b, 54a vorhanden; Frage „What did the IMCO/LIBE compromise amendments change in Article 5?“ nutzt Stufe committee und zeigt Änderungen.</t>
+        </is>
+      </c>
+      <c r="G23" s="22" t="inlineStr">
+        <is>
+          <t>Backend · Legal · Daten</t>
+        </is>
+      </c>
+      <c r="H23" s="22" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="I23" s="22" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
+        </is>
+      </c>
+      <c r="J23" s="22" t="inlineStr">
+        <is>
+          <t>Tests 86 passed; ingest_legal mit Platzhaltern für Qdrant/Neo4j/LLM durchgelaufen (2269 Text Units). Einlesen per Docker mit -e OPENROUTER_API_KEY steht aus. Plenarposition 14.6.2023, allgemeine Ausrichtung des Rates, Verordnung 2024/1689 und konsolidierte Fassung fehlen noch.</t>
         </is>
       </c>
     </row>
@@ -3300,7 +3384,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="130" customWidth="1" style="10" min="1" max="1"/>
@@ -3369,6 +3453,13 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>Release 3.1.0 (29.10.2026, Minor): REQ-43 (Kompromissänderungen IMCO/LIBE als Teilfassung des AI Act) vorbereitet und offline geprüft; Einlesen per Docker ausstehend. Release Notes: CHANGELOG.md, Abschnitt [3.1.0].</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
ALITA v3.1.1 – the adopted AI Act from the Official Journal (REQ-44)
- Official Journal PDFs: footnotes after the page footer are dropped
  (no longer recitals), SECTION headings kept, "Article 49" lines after
  the first annex are references, "Article 58. The Board …" is a reference
- Applicability: the rule naming a component beats the rule for its
  chapter (Art. 101 vs Chapter XII, Art. 113)
- AI Act: Regulation (EU) 2024/1689 as version 3; tests 88 passed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiuZbjdoe5Dn8qVgxqM
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -553,7 +553,7 @@
     <row r="2" ht="15" customHeight="1" s="11">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>Stand: Release 3.1.0 vom 29.10.2026 · REQ-01 – REQ-21 aus dem Review von 2.0.0, REQ-22 – REQ-34 aus der Sitzung vom 17.10.2026 (inkl. Feedback von Dustin), REQ-35 – REQ-43 aus der Sitzung vom 29.10.2026</t>
+          <t>Stand: Release 3.1.1 vom 29.10.2026 · REQ-01 – REQ-21 aus dem Review von 2.0.0, REQ-22 – REQ-34 aus der Sitzung vom 17.10.2026 (inkl. Feedback von Dustin), REQ-35 – REQ-44 aus der Sitzung vom 29.10.2026</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -2116,6 +2116,38 @@
       <c r="F44" s="22" t="inlineStr">
         <is>
           <t>Datei abgelegt, _legal.yaml: Fassung 2 von 4, Stufe „committee“, partial: true. Neu: Teilfassungen (merge_partial – fehlende Teile unverändert aus der Vorfassung, keine Streichungen), Stufe committee im Planer, Parser für Kompromissblöcke CA 1–12, Artikelnummern „54 a“/„28(a)“, Erwägungsgründe „(65a)“, Vergleich nur über Buchstaben/Ziffern (cmp_key). Offline geprüft: 104 Artikel (24 neu), 129 Erwägungsgründe, 0 gestrichen, kleinste Änderungen echt (250 000 → 750 000 EUR, user → deployer). Einlesen per Docker steht aus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" s="11">
+      <c r="A45" s="22" t="inlineStr">
+        <is>
+          <t>REQ-44</t>
+        </is>
+      </c>
+      <c r="B45" s="22" t="inlineStr">
+        <is>
+          <t>Finale Fassung des AI Act: Verordnung (EU) 2024/1689 aus dem Amtsblatt</t>
+        </is>
+      </c>
+      <c r="C45" s="22" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
+        </is>
+      </c>
+      <c r="D45" s="22" t="inlineStr">
+        <is>
+          <t>3.1.1</t>
+        </is>
+      </c>
+      <c r="E45" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 29.10.2026</t>
+        </is>
+      </c>
+      <c r="F45" s="22" t="inlineStr">
+        <is>
+          <t>Datei als 2024-07-12_Regulation-2024-1689_OJ.pdf abgelegt (Fassung 3 von 4, Stufe adopted, in Kraft 1.8.2024, Anwendung nach Art. 113). Parser für Amtsblatt-PDFs korrigiert: Fußnoten nicht mehr als Erwägungsgründe (236 → 180), Abschnitte erhalten (8 → 16), Verweise in Anhängen keine Artikel (115 → 113); Anwendungsregel für Art. 101 schlägt Kapitel XII. Offline geprüft: Struktur exakt wie die Verordnung, Anwendungsdaten Art. 5, 6(1), 50, 53, 78, 99, 101 korrekt. Einlesen per Docker steht aus.</t>
         </is>
       </c>
     </row>
@@ -2150,7 +2182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -3357,6 +3389,58 @@
       <c r="J23" s="22" t="inlineStr">
         <is>
           <t>Tests 86 passed; ingest_legal mit Platzhaltern für Qdrant/Neo4j/LLM durchgelaufen (2269 Text Units). Einlesen per Docker mit -e OPENROUTER_API_KEY steht aus. Plenarposition 14.6.2023, allgemeine Ausrichtung des Rates, Verordnung 2024/1689 und konsolidierte Fassung fehlen noch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" s="11">
+      <c r="A24" s="22" t="inlineStr">
+        <is>
+          <t>REQ-44</t>
+        </is>
+      </c>
+      <c r="B24" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C24" s="22" t="inlineStr">
+        <is>
+          <t>3.1.1</t>
+        </is>
+      </c>
+      <c r="D24" s="22" t="inlineStr">
+        <is>
+          <t>uind jetzt kommt das finale gesetz dazhu [OJ_L_202401689_EN_TXT.pdf]</t>
+        </is>
+      </c>
+      <c r="E24" s="22" t="inlineStr">
+        <is>
+          <t>Das Legal project „EU-AI-Act“ MUSS die im Amtsblatt veröffentlichte Verordnung (EU) 2024/1689 als geltende Fassung (in Kraft ab 1.8.2024) führen, mit den Anwendungsdaten nach Art. 113 je Bestimmung. Fußnoten DÜRFEN NICHT als Erwägungsgründe gelten; Verweise in Anhängen DÜRFEN NICHT als Artikel gelten.</t>
+        </is>
+      </c>
+      <c r="F24" s="22" t="inlineStr">
+        <is>
+          <t>Nach „ingest legal“: drei Fassungen, Verordnung aktuell; 180 Erwägungsgründe, 113 Artikel, 13 Kapitel mit 16 Abschnitten, 13 Anhänge; Art. 5 anwendbar ab 2.2.2025, Art. 6(1) ab 2.8.2027, Art. 101 ab 2.8.2026, Kapitel V ab 2.8.2025; Frage ohne Datum nutzt die Verordnung.</t>
+        </is>
+      </c>
+      <c r="G24" s="22" t="inlineStr">
+        <is>
+          <t>Backend · Legal · Daten</t>
+        </is>
+      </c>
+      <c r="H24" s="22" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="I24" s="22" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
+        </is>
+      </c>
+      <c r="J24" s="22" t="inlineStr">
+        <is>
+          <t>Tests 88 passed; ingest_legal mit Platzhaltern für Qdrant/Neo4j/LLM durchgelaufen (3 Fassungen, 5270 Text Units). Einlesen per Docker mit -e OPENROUTER_API_KEY steht aus. Konsolidierte Fassung (Digital Omnibus) fehlt noch.</t>
         </is>
       </c>
     </row>
@@ -3384,7 +3468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="130" customWidth="1" style="10" min="1" max="1"/>
@@ -3460,6 +3544,13 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="24" t="inlineStr">
+        <is>
+          <t>Release 3.1.1 (29.10.2026, Patch): REQ-44 (Verordnung (EU) 2024/1689 aus dem Amtsblatt als dritte Fassung) vorbereitet und offline geprüft; Einlesen per Docker ausstehend. Release Notes: CHANGELOG.md, Abschnitt [3.1.1].</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
ALITA v3.2.0 – applying an amending act: Digital Omnibus on AI (REQ-45)
- app/legal_amend.py: splits the amending article into instructions
  (target, operation, quoted text) and applies them to the previous
  version; report per instruction (applied / approximate / not_applied)
- _legal.yaml: apply_amendments; AI Act version 4 = consolidated version
  after Regulation (EU) 2026/1744 (63 of 72 exact, 5 approximate, 4 open)
- Paragraph numbers "1a."; OJ footer detection needs a page counter
- Document details show the amendment report; tests 89 passed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiuZbjdoe5Dn8qVgxqM
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -553,7 +553,7 @@
     <row r="2" ht="15" customHeight="1" s="11">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>Stand: Release 3.1.1 vom 29.10.2026 · REQ-01 – REQ-21 aus dem Review von 2.0.0, REQ-22 – REQ-34 aus der Sitzung vom 17.10.2026 (inkl. Feedback von Dustin), REQ-35 – REQ-44 aus der Sitzung vom 29.10.2026</t>
+          <t>Stand: Release 3.2.0 vom 29.10.2026 · REQ-01 – REQ-21 aus dem Review von 2.0.0, REQ-22 – REQ-34 aus der Sitzung vom 17.10.2026 (inkl. Feedback von Dustin), REQ-35 – REQ-45 aus der Sitzung vom 29.10.2026</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -2148,6 +2148,38 @@
       <c r="F45" s="22" t="inlineStr">
         <is>
           <t>Datei als 2024-07-12_Regulation-2024-1689_OJ.pdf abgelegt (Fassung 3 von 4, Stufe adopted, in Kraft 1.8.2024, Anwendung nach Art. 113). Parser für Amtsblatt-PDFs korrigiert: Fußnoten nicht mehr als Erwägungsgründe (236 → 180), Abschnitte erhalten (8 → 16), Verweise in Anhängen keine Artikel (115 → 113); Anwendungsregel für Art. 101 schlägt Kapitel XII. Offline geprüft: Struktur exakt wie die Verordnung, Anwendungsdaten Art. 5, 6(1), 50, 53, 78, 99, 101 korrekt. Einlesen per Docker steht aus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" s="11">
+      <c r="A46" s="22" t="inlineStr">
+        <is>
+          <t>REQ-45</t>
+        </is>
+      </c>
+      <c r="B46" s="22" t="inlineStr">
+        <is>
+          <t>Digital Omnibus on AI (Verordnung (EU) 2026/1744) im Projekt AI Act</t>
+        </is>
+      </c>
+      <c r="C46" s="22" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
+        </is>
+      </c>
+      <c r="D46" s="22" t="inlineStr">
+        <is>
+          <t>3.2.0</t>
+        </is>
+      </c>
+      <c r="E46" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 29.10.2026</t>
+        </is>
+      </c>
+      <c r="F46" s="22" t="inlineStr">
+        <is>
+          <t>Datei als 2026-07-24_Regulation-2026-1744_Digital-Omnibus_OJ.pdf abgelegt; _legal.yaml Fassung 4 (consolidated, in Kraft 27.7.2026, apply_amendments: Regulation (EU) 2024/1689, Anwendungsdaten des geänderten Art. 113). Neu: app/legal_amend.py wendet die 72 Änderungsbefehle auf Fassung 3 an – 63 exakt, 5 angenähert (erster Unterabsatz/Einleitung), 4 offen gemeldet (spätere Unterabsätze, Punkte in Anhängen); neue Art. 4a, 60a, 75a–75d, Anhang XIV; Bericht je Befehl in den Dokumentdetails. Einlesen per Docker steht aus.</t>
         </is>
       </c>
     </row>
@@ -2182,7 +2214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -3441,6 +3473,58 @@
       <c r="J24" s="22" t="inlineStr">
         <is>
           <t>Tests 88 passed; ingest_legal mit Platzhaltern für Qdrant/Neo4j/LLM durchgelaufen (3 Fassungen, 5270 Text Units). Einlesen per Docker mit -e OPENROUTER_API_KEY steht aus. Konsolidierte Fassung (Digital Omnibus) fehlt noch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" s="11">
+      <c r="A25" s="22" t="inlineStr">
+        <is>
+          <t>REQ-45</t>
+        </is>
+      </c>
+      <c r="B25" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C25" s="22" t="inlineStr">
+        <is>
+          <t>3.2.0</t>
+        </is>
+      </c>
+      <c r="D25" s="22" t="inlineStr">
+        <is>
+          <t>jetzt dazu im projekt der omnibus [OJ_L_202601744_EN_TXT.pdf]</t>
+        </is>
+      </c>
+      <c r="E25" s="22" t="inlineStr">
+        <is>
+          <t>Das Legal project „EU-AI-Act“ MUSS die Änderungen des Digital Omnibus on AI (Verordnung (EU) 2026/1744) als neue geltende Fassung ab 27.7.2026 führen. Da das Dokument eine Änderungsverordnung ist, MUSS ALITA die Änderungsbefehle auf die Verordnung 2024/1689 anwenden; Befehle, die nicht sicher angewendet werden können, MÜSSEN offen gemeldet werden und DÜRFEN NICHT stillschweigend fehlen.</t>
+        </is>
+      </c>
+      <c r="F25" s="22" t="inlineStr">
+        <is>
+          <t>Nach „ingest legal“: vier Fassungen in einem Projekt; Verordnung 2024 gilt bis 26.7.2026, konsolidierte Fassung ab 27.7.2026; Art. 4a, 60a, 75a–75d und Anhang XIV vorhanden; Art. 10(5) gestrichen; Art. 5(1)(ba) anwendbar ab 2.12.2026, Kapitel III Abschnitte 1–3 ab 2.12.2027, Art. 6(1) ab 2.8.2028; Dokumentdetails zeigen 63/72 angewendet und die offenen Befehle.</t>
+        </is>
+      </c>
+      <c r="G25" s="22" t="inlineStr">
+        <is>
+          <t>Backend · Legal · Daten</t>
+        </is>
+      </c>
+      <c r="H25" s="22" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="I25" s="22" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
+        </is>
+      </c>
+      <c r="J25" s="22" t="inlineStr">
+        <is>
+          <t>Tests 89 passed; ingest_legal mit Platzhaltern für Qdrant/Neo4j/LLM durchgelaufen (4 Fassungen, 6318 Text Units). Einlesen per Docker mit -e OPENROUTER_API_KEY steht aus. Offen: 2 spätere Unterabsätze und 2 Anhangpunkte; zwei Daten für Kapitel III (Anhang III / Anhang I) auf je einen Teil abgebildet.</t>
         </is>
       </c>
     </row>
@@ -3468,7 +3552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="130" customWidth="1" style="10" min="1" max="1"/>
@@ -3551,6 +3635,13 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="24" t="inlineStr">
+        <is>
+          <t>Release 3.2.0 (29.10.2026, Minor): REQ-45 (Digital Omnibus on AI als vierte Fassung, Änderungsbefehle automatisch angewendet) vorbereitet und offline geprüft; Einlesen per Docker ausstehend. Release Notes: CHANGELOG.md, Abschnitt [3.2.0].</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
ALITA v3.2.1 – Commission guidelines (REQ-46)
- Parser for Commission guidelines: sections I.-III. (sec_II), headings
  "1." / "5.1.", margin numbers "(13)" (rn_13, "Para. 13"), footnote
  blocks left out (only for documents with bracketed margin numbers)
- EU AI Act: Guidelines on the AI system definition, C(2025) 5053 final,
  as the first legal guideline; tests 90 passed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiuZbjdoe5Dn8qVgxqM
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -553,7 +553,7 @@
     <row r="2" ht="15" customHeight="1" s="11">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>Stand: Release 3.2.0 vom 29.10.2026 · REQ-01 – REQ-21 aus dem Review von 2.0.0, REQ-22 – REQ-34 aus der Sitzung vom 17.10.2026 (inkl. Feedback von Dustin), REQ-35 – REQ-45 aus der Sitzung vom 29.10.2026</t>
+          <t>Stand: Release 3.2.1 vom 29.10.2026 · REQ-01 – REQ-21 aus dem Review von 2.0.0, REQ-22 – REQ-34 aus der Sitzung vom 17.10.2026 (inkl. Feedback von Dustin), REQ-35 – REQ-46 aus der Sitzung vom 29.10.2026</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -2180,6 +2180,38 @@
       <c r="F46" s="22" t="inlineStr">
         <is>
           <t>Datei als 2026-07-24_Regulation-2026-1744_Digital-Omnibus_OJ.pdf abgelegt; _legal.yaml Fassung 4 (consolidated, in Kraft 27.7.2026, apply_amendments: Regulation (EU) 2024/1689, Anwendungsdaten des geänderten Art. 113). Neu: app/legal_amend.py wendet die 72 Änderungsbefehle auf Fassung 3 an – 63 exakt, 5 angenähert (erster Unterabsatz/Einleitung), 4 offen gemeldet (spätere Unterabsätze, Punkte in Anhängen); neue Art. 4a, 60a, 75a–75d, Anhang XIV; Bericht je Befehl in den Dokumentdetails. Einlesen per Docker steht aus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" s="11">
+      <c r="A47" s="22" t="inlineStr">
+        <is>
+          <t>REQ-46</t>
+        </is>
+      </c>
+      <c r="B47" s="22" t="inlineStr">
+        <is>
+          <t>Legal guideline: Leitlinien der Kommission zur Definition eines KI-Systems (C(2025) 5053)</t>
+        </is>
+      </c>
+      <c r="C47" s="22" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
+        </is>
+      </c>
+      <c r="D47" s="22" t="inlineStr">
+        <is>
+          <t>3.2.1</t>
+        </is>
+      </c>
+      <c r="E47" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 29.10.2026</t>
+        </is>
+      </c>
+      <c r="F47" s="22" t="inlineStr">
+        <is>
+          <t>Datei und _legal.yaml in research/EUAIA/guidelines/ (Stufe published, gültig ab 29.7.2025). Parser für Kommissionsleitlinien: Abschnitte I.–III. (sec_II), Gliederung 1./5.1., Randnummern (1)–(64) als rn_n („Para. 13“), Fußnotenblöcke ausgelassen; ISO-Normen nicht betroffen. Offline geprüft: 3 Abschnitte, 9 Gliederungspunkte, 64 Randnummern, 138 Text Units. Einlesen per Docker steht aus.</t>
         </is>
       </c>
     </row>
@@ -2214,7 +2246,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -3525,6 +3557,58 @@
       <c r="J25" s="22" t="inlineStr">
         <is>
           <t>Tests 89 passed; ingest_legal mit Platzhaltern für Qdrant/Neo4j/LLM durchgelaufen (4 Fassungen, 6318 Text Units). Einlesen per Docker mit -e OPENROUTER_API_KEY steht aus. Offen: 2 spätere Unterabsätze und 2 Anhangpunkte; zwei Daten für Kapitel III (Anhang III / Anhang I) auf je einen Teil abgebildet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" s="11">
+      <c r="A26" s="22" t="inlineStr">
+        <is>
+          <t>REQ-46</t>
+        </is>
+      </c>
+      <c r="B26" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C26" s="22" t="inlineStr">
+        <is>
+          <t>3.2.1</t>
+        </is>
+      </c>
+      <c r="D26" s="22" t="inlineStr">
+        <is>
+          <t>und jetzt kommt eine legal guideline [Commission_Guidelines_on_the_definition_of_an_artificial_intelligence_system … .PDF]</t>
+        </is>
+      </c>
+      <c r="E26" s="22" t="inlineStr">
+        <is>
+          <t>Die Leitlinien der Kommission zur Definition eines KI-Systems MÜSSEN als Legal guideline in der Datenbank „EU AI Act“ geführt werden, gegliedert nach Abschnitten, Gliederungspunkten und Randnummern, zitierbar als „Para. n“. Fußnoten DÜRFEN NICHT als Gliederung oder Randnummer gelten.</t>
+        </is>
+      </c>
+      <c r="F26" s="22" t="inlineStr">
+        <is>
+          <t>Nach „ingest guideline /research/EUAIA/guidelines“: ein Dokument vom Typ Legal guideline (▲) in EU AI Act, gültig ab 29.7.2025; 64 Randnummern; Frage „What do the Commission guidelines say about adaptiveness?“ nennt Randnummern aus Abschnitt II.3.</t>
+        </is>
+      </c>
+      <c r="G26" s="22" t="inlineStr">
+        <is>
+          <t>Backend · Legal · Daten</t>
+        </is>
+      </c>
+      <c r="H26" s="22" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="I26" s="22" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
+        </is>
+      </c>
+      <c r="J26" s="22" t="inlineStr">
+        <is>
+          <t>Tests 90 passed; ingest_legal als Legal guideline mit Platzhaltern durchgelaufen. Einlesen per Docker mit -e OPENROUTER_API_KEY steht aus. Offen: Verknüpfung der Leitlinie mit Art. 3(1) im Graphen.</t>
         </is>
       </c>
     </row>
@@ -3552,7 +3636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="130" customWidth="1" style="10" min="1" max="1"/>
@@ -3642,6 +3726,13 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="24" t="inlineStr">
+        <is>
+          <t>Release 3.2.1 (29.10.2026, Patch): REQ-46 (Leitlinien der Kommission zur Definition eines KI-Systems als erste Legal guideline) vorbereitet und offline geprüft; Einlesen per Docker ausstehend. Release Notes: CHANGELOG.md, Abschnitt [3.2.1].</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
ALITA v3.2.2 – guidelines on prohibited AI practices (REQ-47)
- Tables of contents (dot leaders, wrapped entries) are skipped
- Commission guidelines: headings must continue the outline, margin
  numbers must follow each other; headings may wrap after a comma or
  start with a quotation mark or bracket
- EU AI Act: Guidelines on prohibited AI practices, C(2025) 5052 final,
  as the second legal guideline (114 headings, 433 margin numbers)
- Tests 91 passed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiuZbjdoe5Dn8qVgxqM
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -553,7 +553,7 @@
     <row r="2" ht="15" customHeight="1" s="11">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>Stand: Release 3.2.1 vom 29.10.2026 · REQ-01 – REQ-21 aus dem Review von 2.0.0, REQ-22 – REQ-34 aus der Sitzung vom 17.10.2026 (inkl. Feedback von Dustin), REQ-35 – REQ-46 aus der Sitzung vom 29.10.2026</t>
+          <t>Stand: Release 3.2.2 vom 29.10.2026 · REQ-01 – REQ-21 aus dem Review von 2.0.0, REQ-22 – REQ-34 aus der Sitzung vom 17.10.2026 (inkl. Feedback von Dustin), REQ-35 – REQ-47 aus der Sitzung vom 29.10.2026</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -2212,6 +2212,38 @@
       <c r="F47" s="22" t="inlineStr">
         <is>
           <t>Datei und _legal.yaml in research/EUAIA/guidelines/ (Stufe published, gültig ab 29.7.2025). Parser für Kommissionsleitlinien: Abschnitte I.–III. (sec_II), Gliederung 1./5.1., Randnummern (1)–(64) als rn_n („Para. 13“), Fußnotenblöcke ausgelassen; ISO-Normen nicht betroffen. Offline geprüft: 3 Abschnitte, 9 Gliederungspunkte, 64 Randnummern, 138 Text Units. Einlesen per Docker steht aus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" s="11">
+      <c r="A48" s="22" t="inlineStr">
+        <is>
+          <t>REQ-47</t>
+        </is>
+      </c>
+      <c r="B48" s="22" t="inlineStr">
+        <is>
+          <t>Zweite Legal guideline: Leitlinien der Kommission zu verbotenen KI-Praktiken (C(2025) 5052)</t>
+        </is>
+      </c>
+      <c r="C48" s="22" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
+        </is>
+      </c>
+      <c r="D48" s="22" t="inlineStr">
+        <is>
+          <t>3.2.2</t>
+        </is>
+      </c>
+      <c r="E48" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 29.10.2026</t>
+        </is>
+      </c>
+      <c r="F48" s="22" t="inlineStr">
+        <is>
+          <t>Datei in research/EUAIA/guidelines/, zweiter Eintrag in der _legal.yaml (published, gültig ab 29.7.2025). Parser: Inhaltsverzeichnis übersprungen, Gliederung und Randnummern müssen fortlaufen (Aufzählungen, zitierte Artikel, „(2022) doi:…“ bleiben Text), Überschriften mit Komma-Umbruch, Anführungszeichen oder Klammer. Offline geprüft: 114 Gliederungspunkte, 433 Randnummern lückenlos, keine Dubletten. Einlesen per Docker steht aus.</t>
         </is>
       </c>
     </row>
@@ -2246,7 +2278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -3609,6 +3641,58 @@
       <c r="J26" s="22" t="inlineStr">
         <is>
           <t>Tests 90 passed; ingest_legal als Legal guideline mit Platzhaltern durchgelaufen. Einlesen per Docker mit -e OPENROUTER_API_KEY steht aus. Offen: Verknüpfung der Leitlinie mit Art. 3(1) im Graphen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" s="11">
+      <c r="A27" s="22" t="inlineStr">
+        <is>
+          <t>REQ-47</t>
+        </is>
+      </c>
+      <c r="B27" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C27" s="22" t="inlineStr">
+        <is>
+          <t>3.2.2</t>
+        </is>
+      </c>
+      <c r="D27" s="22" t="inlineStr">
+        <is>
+          <t>und noch ein legal guideline [Guidelines_on_prohibited_artificial_intelligence_practices … .PDF]</t>
+        </is>
+      </c>
+      <c r="E27" s="22" t="inlineStr">
+        <is>
+          <t>Die Leitlinien der Kommission zu verbotenen KI-Praktiken MÜSSEN als zweite Legal guideline in „EU AI Act“ geführt werden; Inhaltsverzeichnis, Aufzählungen im Text und zitierte Bestimmungen DÜRFEN NICHT als Gliederung gelten; alle Randnummern MÜSSEN vollständig und eindeutig sein.</t>
+        </is>
+      </c>
+      <c r="F27" s="22" t="inlineStr">
+        <is>
+          <t>Nach „ingest guideline /research/EUAIA/guidelines“: zwei Legal guidelines; diese mit 433 Randnummern ohne Dubletten und 114 Gliederungspunkten; Frage „What do the guidelines say about social scoring?“ nennt Randnummern aus Kapitel 4.</t>
+        </is>
+      </c>
+      <c r="G27" s="22" t="inlineStr">
+        <is>
+          <t>Backend · Legal · Daten</t>
+        </is>
+      </c>
+      <c r="H27" s="22" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="I27" s="22" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
+        </is>
+      </c>
+      <c r="J27" s="22" t="inlineStr">
+        <is>
+          <t>Tests 91 passed; ingest_legal für beide Leitlinien mit Platzhaltern durchgelaufen. Einlesen per Docker mit -e OPENROUTER_API_KEY steht aus.</t>
         </is>
       </c>
     </row>
@@ -3636,7 +3720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="130" customWidth="1" style="10" min="1" max="1"/>
@@ -3733,6 +3817,13 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="24" t="inlineStr">
+        <is>
+          <t>Release 3.2.2 (29.10.2026, Patch): REQ-47 (Leitlinien der Kommission zu verbotenen KI-Praktiken als zweite Legal guideline) vorbereitet und offline geprüft; Einlesen per Docker ausstehend. Release Notes: CHANGELOG.md, Abschnitt [3.2.2].</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
ALITA v3.3.0 – new document class "Guidance & FAQ" (REQ-48)
- Document type guidance: Q&A pages, FAQs, factsheets of authorities
  (not binding, no reference number), separate from legal guidelines;
  folders guidance/ faq/ faqs/, CLI "ingest guidance", upload, chip "FAQ",
  olive triangle, fabio:WebPage / bibo:Webpage, clustering unit
- parse_faq: topics (tp_n) and questions (q_n.m, "Q 2.1"); stage snapshot
- EU AI Act: "AI Literacy – Questions & Answers" (AI Office, 29.10.2026)
- Tests 92 passed; UI checked against the mock API

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiuZbjdoe5Dn8qVgxqM
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -553,7 +553,7 @@
     <row r="2" ht="15" customHeight="1" s="11">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>Stand: Release 3.2.2 vom 29.10.2026 · REQ-01 – REQ-21 aus dem Review von 2.0.0, REQ-22 – REQ-34 aus der Sitzung vom 17.10.2026 (inkl. Feedback von Dustin), REQ-35 – REQ-47 aus der Sitzung vom 29.10.2026</t>
+          <t>Stand: Release 3.3.0 vom 29.10.2026 · REQ-01 – REQ-21 aus dem Review von 2.0.0, REQ-22 – REQ-34 aus der Sitzung vom 17.10.2026 (inkl. Feedback von Dustin), REQ-35 – REQ-48 aus der Sitzung vom 29.10.2026</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -2244,6 +2244,38 @@
       <c r="F48" s="22" t="inlineStr">
         <is>
           <t>Datei in research/EUAIA/guidelines/, zweiter Eintrag in der _legal.yaml (published, gültig ab 29.7.2025). Parser: Inhaltsverzeichnis übersprungen, Gliederung und Randnummern müssen fortlaufen (Aufzählungen, zitierte Artikel, „(2022) doi:…“ bleiben Text), Überschriften mit Komma-Umbruch, Anführungszeichen oder Klammer. Offline geprüft: 114 Gliederungspunkte, 433 Randnummern lückenlos, keine Dubletten. Einlesen per Docker steht aus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" s="11">
+      <c r="A49" s="22" t="inlineStr">
+        <is>
+          <t>REQ-48</t>
+        </is>
+      </c>
+      <c r="B49" s="22" t="inlineStr">
+        <is>
+          <t>Neue Dokumentklasse „Guidance &amp; FAQ“ für EU AI Act (erstes Dokument: AI Literacy – Questions &amp; Answers)</t>
+        </is>
+      </c>
+      <c r="C49" s="22" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
+        </is>
+      </c>
+      <c r="D49" s="22" t="inlineStr">
+        <is>
+          <t>3.3.0</t>
+        </is>
+      </c>
+      <c r="E49" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 29.10.2026</t>
+        </is>
+      </c>
+      <c r="F49" s="22" t="inlineStr">
+        <is>
+          <t>Neuer Typ guidance („Guidance &amp; FAQ“): Q&amp;A-Seiten, FAQs, Factsheets von Behörden ohne Aktenzeichen, unverbindlich – abgegrenzt von förmlichen Legal guidelines. Ordner research/&lt;DB&gt;/guidance/, CLI ingest guidance, Upload, Filter-Chip „FAQ“, ▲ olivgrün, fabio:WebPage/bibo:Webpage. Parser: Themen tp_n und Fragen q_n.m („Q 2.1“), Stufe snapshot für Webseitenstände. Erstes Dokument: AI Literacy Q&amp;A (digital-strategy.ec.europa.eu, Stand 29.10.2026): 5 Themen, 34 Fragen. UI im Mock geprüft. Einlesen per Docker steht aus.</t>
         </is>
       </c>
     </row>
@@ -2278,7 +2310,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -3693,6 +3725,58 @@
       <c r="J27" s="22" t="inlineStr">
         <is>
           <t>Tests 91 passed; ingest_legal für beide Leitlinien mit Platzhaltern durchgelaufen. Einlesen per Docker mit -e OPENROUTER_API_KEY steht aus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" s="11">
+      <c r="A28" s="22" t="inlineStr">
+        <is>
+          <t>REQ-48</t>
+        </is>
+      </c>
+      <c r="B28" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C28" s="22" t="inlineStr">
+        <is>
+          <t>3.3.0</t>
+        </is>
+      </c>
+      <c r="D28" s="22" t="inlineStr">
+        <is>
+          <t>jetzt kommet eher etwas anderes aber ich weiß nicht wie ich das nenne soll mach du eine neue dokumentenklasse auf für die eu ai act db [node_13629_printable_pdf.pdf – AI Literacy - Questions &amp; Answers]</t>
+        </is>
+      </c>
+      <c r="E28" s="22" t="inlineStr">
+        <is>
+          <t>Es MUSS eine eigene Dokumentklasse für unverbindliche Erläuterungen von Behörden (Q&amp;A-Seiten, FAQs, Factsheets) geben, getrennt von förmlichen Leitlinien; solche Dokumente MÜSSEN nach Themen und Fragen gegliedert und als „Q n.m“ zitierbar sein; Stände einer Webseite SOLLEN als Fassungen über die Zeit geführt werden.</t>
+        </is>
+      </c>
+      <c r="F28" s="22" t="inlineStr">
+        <is>
+          <t>Nach „ingest guidance /research/EUAIA/guidance“: Dokument „AI Literacy – Questions &amp; Answers“ vom Typ Guidance &amp; FAQ (▲, Chip „FAQ“) in EU AI Act, Stufe „Web page snapshot“ ab 29.10.2026; 5 Themen, 34 Fragen; Frage „Is AI training mandatory under Article 4?“ nennt Q 2.3 als Quelle.</t>
+        </is>
+      </c>
+      <c r="G28" s="22" t="inlineStr">
+        <is>
+          <t>Backend · Frontend · Legal · Daten</t>
+        </is>
+      </c>
+      <c r="H28" s="22" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="I28" s="22" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
+        </is>
+      </c>
+      <c r="J28" s="22" t="inlineStr">
+        <is>
+          <t>Name gewählt von Claude: „Guidance &amp; FAQ“ (guidance). Tests 92 passed; ingest_legal als guidance mit Platzhaltern durchgelaufen (40 Bestandteile); Oberfläche mit Mock-API geprüft. Einlesen per Docker mit -e OPENROUTER_API_KEY steht aus.</t>
         </is>
       </c>
     </row>
@@ -3720,7 +3804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="130" customWidth="1" style="10" min="1" max="1"/>
@@ -3824,6 +3908,13 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="24" t="inlineStr">
+        <is>
+          <t>Release 3.3.0 (29.10.2026, Minor): REQ-48 (neue Dokumentklasse „Guidance &amp; FAQ“, erstes Dokument AI Literacy Q&amp;A) vorbereitet und offline geprüft; Einlesen per Docker ausstehend. Release Notes: CHANGELOG.md, Abschnitt [3.3.0].</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
ALITA v3.3.1 – first standard, licence stamps removed (REQ-49)
- extract.strip_licence_stamps: personal download stamps of standards
  (name, customer number, download ID, time) never reach index or LLM
- Standards: terms as parts (type term), annex status behind the title,
  annex clauses C.1.2.1, numbered table rows in annexes stay text
- EU AI Act: DIN SPEC 92005:2024-03 as the first standard; tests 93 passed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiuZbjdoe5Dn8qVgxqM
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -553,7 +553,7 @@
     <row r="2" ht="15" customHeight="1" s="11">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>Stand: Release 3.3.0 vom 29.10.2026 · REQ-01 – REQ-21 aus dem Review von 2.0.0, REQ-22 – REQ-34 aus der Sitzung vom 17.10.2026 (inkl. Feedback von Dustin), REQ-35 – REQ-48 aus der Sitzung vom 29.10.2026</t>
+          <t>Stand: Release 3.3.1 vom 30.10.2026 · REQ-01 – REQ-21 aus dem Review von 2.0.0, REQ-22 – REQ-34 aus der Sitzung vom 17.10.2026 (inkl. Feedback von Dustin), REQ-35 – REQ-49 aus der Sitzung vom 29.10.2026</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -2276,6 +2276,38 @@
       <c r="F49" s="22" t="inlineStr">
         <is>
           <t>Neuer Typ guidance („Guidance &amp; FAQ“): Q&amp;A-Seiten, FAQs, Factsheets von Behörden ohne Aktenzeichen, unverbindlich – abgegrenzt von förmlichen Legal guidelines. Ordner research/&lt;DB&gt;/guidance/, CLI ingest guidance, Upload, Filter-Chip „FAQ“, ▲ olivgrün, fabio:WebPage/bibo:Webpage. Parser: Themen tp_n und Fragen q_n.m („Q 2.1“), Stufe snapshot für Webseitenstände. Erstes Dokument: AI Literacy Q&amp;A (digital-strategy.ec.europa.eu, Stand 29.10.2026): 5 Themen, 34 Fragen. UI im Mock geprüft. Einlesen per Docker steht aus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" s="11">
+      <c r="A50" s="22" t="inlineStr">
+        <is>
+          <t>REQ-49</t>
+        </is>
+      </c>
+      <c r="B50" s="22" t="inlineStr">
+        <is>
+          <t>Erster Standard: DIN SPEC 92005:2024-03 (Uncertainty quantification in machine learning)</t>
+        </is>
+      </c>
+      <c r="C50" s="22" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
+        </is>
+      </c>
+      <c r="D50" s="22" t="inlineStr">
+        <is>
+          <t>3.3.1</t>
+        </is>
+      </c>
+      <c r="E50" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 29./30.10.2026</t>
+        </is>
+      </c>
+      <c r="F50" s="22" t="inlineStr">
+        <is>
+          <t>Datei und _legal.yaml in research/EUAIA/standards/ (published, ab 1.3.2024). Personalisierte Lizenzstempel (Name, Kundennummer, Download-ID, Zeit) werden beim Auslesen jeder PDF entfernt. Normen: Begriffe als eigene Bestandteile (28), Anhangstatus, Anhang-Gliederung C.1.2.1, Tabellenzeilen in Anhängen als Text. Offline geprüft: kein Stempel, Abschnitte 1–7, 28 Begriffe, Anhänge A–C, 174 Text Units. Lizenz vor dem Einlesen prüfen (Einzelplatzlizenz, externer KI-Dienst).</t>
         </is>
       </c>
     </row>
@@ -2310,7 +2342,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -3777,6 +3809,58 @@
       <c r="J28" s="22" t="inlineStr">
         <is>
           <t>Name gewählt von Claude: „Guidance &amp; FAQ“ (guidance). Tests 92 passed; ingest_legal als guidance mit Platzhaltern durchgelaufen (40 Bestandteile); Oberfläche mit Mock-API geprüft. Einlesen per Docker mit -e OPENROUTER_API_KEY steht aus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" s="11">
+      <c r="A29" s="22" t="inlineStr">
+        <is>
+          <t>REQ-49</t>
+        </is>
+      </c>
+      <c r="B29" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C29" s="22" t="inlineStr">
+        <is>
+          <t>3.3.1</t>
+        </is>
+      </c>
+      <c r="D29" s="22" t="inlineStr">
+        <is>
+          <t>jetzt ein standard [3521675.PDF – DIN SPEC 92005:2024-03]</t>
+        </is>
+      </c>
+      <c r="E29" s="22" t="inlineStr">
+        <is>
+          <t>Die DIN SPEC 92005:2024-03 MUSS als Standard in „EU AI Act“ geführt werden, gegliedert in Abschnitte, Begriffe und Anhänge. Personenbezogene Lizenzstempel des Downloads DÜRFEN NICHT in Index, Graph oder Prompts gelangen.</t>
+        </is>
+      </c>
+      <c r="F29" s="22" t="inlineStr">
+        <is>
+          <t>Nach „ingest standard /research/EUAIA/standards“: Standard „DIN SPEC 92005“ (▲) in EU AI Act; 28 Begriffe (z. B. „uncertainty quantification“), Anhänge A–C; kein Name/keine Kundennummer im Text; Frage „How does DIN SPEC 92005 define aleatoric uncertainty?“ nennt Clause 3.3.</t>
+        </is>
+      </c>
+      <c r="G29" s="22" t="inlineStr">
+        <is>
+          <t>Backend · Legal · Datenschutz · Daten</t>
+        </is>
+      </c>
+      <c r="H29" s="22" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="I29" s="22" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
+        </is>
+      </c>
+      <c r="J29" s="22" t="inlineStr">
+        <is>
+          <t>Tests 93 passed; ingest_legal als standard mit Platzhaltern durchgelaufen (92 Bestandteile). Offen: Lizenz der DIN-Media-Datei für gemeinsame Instanz und externen KI-Dienst prüfen; danach Einlesen per Docker.</t>
         </is>
       </c>
     </row>
@@ -3804,7 +3888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="130" customWidth="1" style="10" min="1" max="1"/>
@@ -3915,6 +3999,13 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="24" t="inlineStr">
+        <is>
+          <t>Release 3.3.1 (30.10.2026, Patch): REQ-49 (DIN SPEC 92005 als erster Standard, Lizenzstempel werden entfernt) vorbereitet und offline geprüft; Lizenz prüfen, dann Einlesen per Docker. Release Notes: CHANGELOG.md, Abschnitt [3.3.1].</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
ALITA v3.3.2 – NIST SP 800-18 Rev. 2 (REQ-50)
- Standards: "Appendix A." counts as an annex; unnumbered "References" /
  "Bibliography" starts a supplement instead of continuing the last clause
- EU AI Act: NIST SP 800-18r2 as the second standard; tests 94 passed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiuZbjdoe5Dn8qVgxqM
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -553,7 +553,7 @@
     <row r="2" ht="15" customHeight="1" s="11">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>Stand: Release 3.3.1 vom 30.10.2026 · REQ-01 – REQ-21 aus dem Review von 2.0.0, REQ-22 – REQ-34 aus der Sitzung vom 17.10.2026 (inkl. Feedback von Dustin), REQ-35 – REQ-49 aus der Sitzung vom 29.10.2026</t>
+          <t>Stand: Release 3.3.2 vom 30.10.2026 · REQ-01 – REQ-21 aus dem Review von 2.0.0, REQ-22 – REQ-34 aus der Sitzung vom 17.10.2026 (inkl. Feedback von Dustin), REQ-35 – REQ-50 aus der Sitzung vom 29.10.2026</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -2308,6 +2308,38 @@
       <c r="F50" s="22" t="inlineStr">
         <is>
           <t>Datei und _legal.yaml in research/EUAIA/standards/ (published, ab 1.3.2024). Personalisierte Lizenzstempel (Name, Kundennummer, Download-ID, Zeit) werden beim Auslesen jeder PDF entfernt. Normen: Begriffe als eigene Bestandteile (28), Anhangstatus, Anhang-Gliederung C.1.2.1, Tabellenzeilen in Anhängen als Text. Offline geprüft: kein Stempel, Abschnitte 1–7, 28 Begriffe, Anhänge A–C, 174 Text Units. Lizenz vor dem Einlesen prüfen (Einzelplatzlizenz, externer KI-Dienst).</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" s="11">
+      <c r="A51" s="22" t="inlineStr">
+        <is>
+          <t>REQ-50</t>
+        </is>
+      </c>
+      <c r="B51" s="22" t="inlineStr">
+        <is>
+          <t>Weiterer Standard: NIST SP 800-18 Rev. 2 (System plans)</t>
+        </is>
+      </c>
+      <c r="C51" s="22" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
+        </is>
+      </c>
+      <c r="D51" s="22" t="inlineStr">
+        <is>
+          <t>3.3.2</t>
+        </is>
+      </c>
+      <c r="E51" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 30.10.2026</t>
+        </is>
+      </c>
+      <c r="F51" s="22" t="inlineStr">
+        <is>
+          <t>Zweiter Eintrag in research/EUAIA/standards/_legal.yaml (published, Juni 2026; frei verfügbar). Parser: „Appendix A.“ als Anhang, „References“/„Bibliography“ als eigene Anlage. Offline geprüft: Abschnitte 1–4.7, References, Anhänge A–D. Erster Upload war versehentlich nochmals die DIN SPEC 92005 (byte-identisch) – dafür nichts geändert. Einlesen per Docker steht aus.</t>
         </is>
       </c>
     </row>
@@ -2342,7 +2374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -3861,6 +3893,58 @@
       <c r="J29" s="22" t="inlineStr">
         <is>
           <t>Tests 93 passed; ingest_legal als standard mit Platzhaltern durchgelaufen (92 Bestandteile). Offen: Lizenz der DIN-Media-Datei für gemeinsame Instanz und externen KI-Dienst prüfen; danach Einlesen per Docker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" s="11">
+      <c r="A30" s="22" t="inlineStr">
+        <is>
+          <t>REQ-50</t>
+        </is>
+      </c>
+      <c r="B30" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C30" s="22" t="inlineStr">
+        <is>
+          <t>3.3.2</t>
+        </is>
+      </c>
+      <c r="D30" s="22" t="inlineStr">
+        <is>
+          <t>nochmal so ein e art standard [3521675.PDF – identisch mit DIN SPEC 92005] / [NIST.SP.800-18r2.pdf]</t>
+        </is>
+      </c>
+      <c r="E30" s="22" t="inlineStr">
+        <is>
+          <t>NIST SP 800-18 Rev. 2 MUSS als weiterer Standard in „EU AI Act“ geführt werden, mit Abschnitten, Anhängen (Appendix A–D) und Literaturverzeichnis als eigenen Bestandteilen. Doppelte Uploads DÜRFEN NICHT zu doppelten Dokumenten führen.</t>
+        </is>
+      </c>
+      <c r="F30" s="22" t="inlineStr">
+        <is>
+          <t>Nach „ingest standard /research/EUAIA/standards“: zwei Standards (DIN SPEC 92005, NIST SP 800-18r2); NIST mit 28 Abschnitten, References und Anhängen A–D; Frage „What does NIST SP 800-18r2 say about consolidated system plans?“ nennt Clause 2.4.</t>
+        </is>
+      </c>
+      <c r="G30" s="22" t="inlineStr">
+        <is>
+          <t>Backend · Legal · Daten</t>
+        </is>
+      </c>
+      <c r="H30" s="22" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="I30" s="22" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
+        </is>
+      </c>
+      <c r="J30" s="22" t="inlineStr">
+        <is>
+          <t>Tests 94 passed; ingest_legal für beide Standards mit Platzhaltern durchgelaufen. Einlesen per Docker mit -e OPENROUTER_API_KEY steht aus (DIN-Lizenz vorher prüfen).</t>
         </is>
       </c>
     </row>
@@ -3888,7 +3972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="130" customWidth="1" style="10" min="1" max="1"/>
@@ -4006,6 +4090,13 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="24" t="inlineStr">
+        <is>
+          <t>Release 3.3.2 (30.10.2026, Patch): REQ-50 (NIST SP 800-18 Rev. 2 als zweiter Standard) vorbereitet und offline geprüft; Einlesen per Docker ausstehend. Release Notes: CHANGELOG.md, Abschnitt [3.3.2].</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
ALITA v3.4.0 – White Paper as accompanying document (REQ-51)
- Project role white_paper ("White paper"), summarised like a manuscript
- _legal.yaml: documents: {file, role, date, title} for accompanying
  documents of a legal project; never taken as versions of the norm
- EU AI Act: White Paper on AI, COM(2020) 65 (19.2.2020); tests 95 passed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiuZbjdoe5Dn8qVgxqM
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -553,7 +553,7 @@
     <row r="2" ht="15" customHeight="1" s="11">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>Stand: Release 3.3.2 vom 30.10.2026 · REQ-01 – REQ-21 aus dem Review von 2.0.0, REQ-22 – REQ-34 aus der Sitzung vom 17.10.2026 (inkl. Feedback von Dustin), REQ-35 – REQ-50 aus der Sitzung vom 29.10.2026</t>
+          <t>Stand: Release 3.4.0 vom 30.10.2026 · REQ-01 – REQ-21 aus dem Review von 2.0.0, REQ-22 – REQ-34 aus der Sitzung vom 17.10.2026 (inkl. Feedback von Dustin), REQ-35 – REQ-51 aus der Sitzung vom 29.10.2026</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -2340,6 +2340,38 @@
       <c r="F51" s="22" t="inlineStr">
         <is>
           <t>Zweiter Eintrag in research/EUAIA/standards/_legal.yaml (published, Juni 2026; frei verfügbar). Parser: „Appendix A.“ als Anhang, „References“/„Bibliography“ als eigene Anlage. Offline geprüft: Abschnitte 1–4.7, References, Anhänge A–D. Erster Upload war versehentlich nochmals die DIN SPEC 92005 (byte-identisch) – dafür nichts geändert. Einlesen per Docker steht aus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" s="11">
+      <c r="A52" s="22" t="inlineStr">
+        <is>
+          <t>REQ-51</t>
+        </is>
+      </c>
+      <c r="B52" s="22" t="inlineStr">
+        <is>
+          <t>Weißbuch zur KI (COM(2020) 65) als White paper im Projekt EU AI Act</t>
+        </is>
+      </c>
+      <c r="C52" s="22" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
+        </is>
+      </c>
+      <c r="D52" s="22" t="inlineStr">
+        <is>
+          <t>3.4.0</t>
+        </is>
+      </c>
+      <c r="E52" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 30.10.2026</t>
+        </is>
+      </c>
+      <c r="F52" s="22" t="inlineStr">
+        <is>
+          <t>Datei im Legal project EU-AI-Act, Eintrag unter documents: in der _legal.yaml (Rolle white_paper, 19.2.2020). Neu: Projektrolle white_paper („White paper“, wird zusammengefasst), Abschnitt documents: für Begleitdokumente (Rolle, Datum, Titel; nie Fassung der Norm). Offline geprüft: Projekt mit 5 Dateien, Weißbuch mit Rolle und Datum. Einlesen per Docker steht aus.</t>
         </is>
       </c>
     </row>
@@ -2374,7 +2406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J30"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -3945,6 +3977,58 @@
       <c r="J30" s="22" t="inlineStr">
         <is>
           <t>Tests 94 passed; ingest_legal für beide Standards mit Platzhaltern durchgelaufen. Einlesen per Docker mit -e OPENROUTER_API_KEY steht aus (DIN-Lizenz vorher prüfen).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" s="11">
+      <c r="A31" s="22" t="inlineStr">
+        <is>
+          <t>REQ-51</t>
+        </is>
+      </c>
+      <c r="B31" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C31" s="22" t="inlineStr">
+        <is>
+          <t>3.4.0</t>
+        </is>
+      </c>
+      <c r="D31" s="22" t="inlineStr">
+        <is>
+          <t>add this paper with is whitepaper [commission-white-paper-artificial-intelligence-feb2020_en.pdf]</t>
+        </is>
+      </c>
+      <c r="E31" s="22" t="inlineStr">
+        <is>
+          <t>Das Weißbuch der Kommission zur KI MUSS als Dokument mit der Rolle „White paper“ im Legal project EU-AI-Act geführt werden, mit seinem Datum (19.2.2020) vor dem Vorschlag; es DARF NICHT als Fassung des Gesetzes gelten.</t>
+        </is>
+      </c>
+      <c r="F31" s="22" t="inlineStr">
+        <is>
+          <t>Nach „ingest legal /research/EUAIA/legal/EU-AI-Act“: Projekt mit 5 Dateien; Weißbuch mit Rolle „White paper“, Datum 19.2.2020, eigener Zusammenfassung; Frage „What did the 2020 White Paper propose and what ended up in the AI Act?“ nennt Weißbuch und Verordnung.</t>
+        </is>
+      </c>
+      <c r="G31" s="22" t="inlineStr">
+        <is>
+          <t>Backend · Legal · Daten</t>
+        </is>
+      </c>
+      <c r="H31" s="22" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="I31" s="22" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
+        </is>
+      </c>
+      <c r="J31" s="22" t="inlineStr">
+        <is>
+          <t>Tests 95 passed; ingest_legal mit Platzhaltern durchgelaufen. Einlesen per Docker mit -e OPENROUTER_API_KEY steht aus.</t>
         </is>
       </c>
     </row>
@@ -3972,7 +4056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="130" customWidth="1" style="10" min="1" max="1"/>
@@ -4097,6 +4181,13 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="24" t="inlineStr">
+        <is>
+          <t>Release 3.4.0 (30.10.2026, Minor): REQ-51 (Weißbuch zur KI als White paper im Legal project) vorbereitet und offline geprüft; Einlesen per Docker ausstehend. Release Notes: CHANGELOG.md, Abschnitt [3.4.0].</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
ALITA v3.5.0 – only "EU AI Act" public, other databases behind a password (REQ-52)
- Without the password the front end shows only the EU AI Act database
  (database bar, documents, projects, clusters, views, people, citations);
  an empty selection sends databases=[EUAIA] to both chats
- Header: field "Password" next to the OpenRouter key, "Lock" button;
  unlock remembered in localStorage
- Display filter only, not access control: the API still serves all databases

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiw6EWVWF8ScrYC2GD7
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -557,7 +557,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="11">
       <c r="A4" s="14" t="inlineStr">
         <is>
@@ -701,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -2372,6 +2371,38 @@
       <c r="F52" s="22" t="inlineStr">
         <is>
           <t>Datei im Legal project EU-AI-Act, Eintrag unter documents: in der _legal.yaml (Rolle white_paper, 19.2.2020). Neu: Projektrolle white_paper („White paper“, wird zusammengefasst), Abschnitt documents: für Begleitdokumente (Rolle, Datum, Titel; nie Fassung der Norm). Offline geprüft: Projekt mit 5 Dateien, Weißbuch mit Rolle und Datum. Einlesen per Docker steht aus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="22" t="inlineStr">
+        <is>
+          <t>REQ-52</t>
+        </is>
+      </c>
+      <c r="B53" s="22" t="inlineStr">
+        <is>
+          <t>Nur „EU AI Act“ öffentlich; übrige Datenbanken erst nach Passwort neben dem OpenRouter-Key</t>
+        </is>
+      </c>
+      <c r="C53" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="D53" s="22" t="inlineStr">
+        <is>
+          <t>3.5.0</t>
+        </is>
+      </c>
+      <c r="E53" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 30.10.2026</t>
+        </is>
+      </c>
+      <c r="F53" s="22" t="inlineStr">
+        <is>
+          <t>Frontend-Filter für alle Ansichten und Chat-Anfragen; Feld „Password“ + „Lock“. Nur Anzeige-Filter, kein API-Schutz. Benötigt Deploy (frontend).</t>
         </is>
       </c>
     </row>
@@ -2406,7 +2437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J32"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -4029,6 +4060,58 @@
       <c r="J31" s="22" t="inlineStr">
         <is>
           <t>Tests 95 passed; ingest_legal mit Platzhaltern durchgelaufen. Einlesen per Docker mit -e OPENROUTER_API_KEY steht aus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="22" t="inlineStr">
+        <is>
+          <t>REQ-52</t>
+        </is>
+      </c>
+      <c r="B32" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C32" s="22" t="inlineStr">
+        <is>
+          <t>3.5.0</t>
+        </is>
+      </c>
+      <c r="D32" s="22" t="inlineStr">
+        <is>
+          <t>Versteck alle Datenbanken außer EU AI Act . Die anderen Datenbanken werden erst dann angezeigt, wenn man neben oprenouter key ein passwort eingibt. Das password ist "password".</t>
+        </is>
+      </c>
+      <c r="E32" s="22" t="inlineStr">
+        <is>
+          <t>Ohne Passwort MUSS die Oberfläche nur die Datenbank „EU AI Act“ anzeigen (Datenbankleiste, Dokumente, Projekte, Cluster, 3D-/Zeitansicht, Personen, Zitationen); die Chats DÜRFEN NICHT in anderen Datenbanken suchen. Die übrigen Datenbanken MÜSSEN nach Eingabe des Passworts in einem Feld neben dem OpenRouter-Key angezeigt werden.</t>
+        </is>
+      </c>
+      <c r="F32" s="22" t="inlineStr">
+        <is>
+          <t>Ohne Passwort: nur „EU AI Act“ in der Datenbankleiste, leere Auswahl sendet databases=[EUAIA]. Falsches Passwort: keine Änderung. Richtiges Passwort + Save: alle neun Datenbanken. „Lock“: wieder nur EU AI Act.</t>
+        </is>
+      </c>
+      <c r="G32" s="22" t="inlineStr">
+        <is>
+          <t>Frontend · Zugriff</t>
+        </is>
+      </c>
+      <c r="H32" s="22" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="I32" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="J32" s="22" t="inlineStr">
+        <is>
+          <t>Frontend-Filter (PUBLIC_DBS, applyDbGate, dbGateFilter, dbScope); Feld „Password“ + „Lock“ im Header; Freischaltung in localStorage. Headless-Browser-Test bestanden. Hinweis: kein Zugriffsschutz – die API liefert weiterhin alle Datenbanken, das Passwort steht im Frontend-Code.</t>
         </is>
       </c>
     </row>
@@ -4056,7 +4139,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="130" customWidth="1" style="10" min="1" max="1"/>
@@ -4181,10 +4264,17 @@
         </is>
       </c>
     </row>
-    <row r="18">
+    <row r="18" s="11">
       <c r="A18" s="24" t="inlineStr">
         <is>
           <t>Release 3.4.0 (30.10.2026, Minor): REQ-51 (Weißbuch zur KI als White paper im Legal project) vorbereitet und offline geprüft; Einlesen per Docker ausstehend. Release Notes: CHANGELOG.md, Abschnitt [3.4.0].</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="24" t="inlineStr">
+        <is>
+          <t>Release 3.5.0 (30.10.2026, Minor): REQ-52 (nur „EU AI Act“ ohne Passwort sichtbar; übrige Datenbanken nach Passwort neben dem OpenRouter-Key).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ALITA v3.5.1 – no "+ Add new data" button in the database bar (REQ-54)
- Removed the button from the database bar; uploads into the existing
  databases remain under Documents → + Upload
- REQ-53 (three papers for EU AI Act) withdrawn by the requester; logged
- User manual and Quick Reference updated; tests 95 passed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiw6EWVWF8ScrYC2GD7
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -700,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -2374,7 +2374,7 @@
         </is>
       </c>
     </row>
-    <row r="53">
+    <row r="53" s="11">
       <c r="A53" s="22" t="inlineStr">
         <is>
           <t>REQ-52</t>
@@ -2403,6 +2403,70 @@
       <c r="F53" s="22" t="inlineStr">
         <is>
           <t>Frontend-Filter für alle Ansichten und Chat-Anfragen; Feld „Password“ + „Lock“. Nur Anzeige-Filter, kein API-Schutz. Benötigt Deploy (frontend).</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" s="11">
+      <c r="A54" s="22" t="inlineStr">
+        <is>
+          <t>REQ-53</t>
+        </is>
+      </c>
+      <c r="B54" s="22" t="inlineStr">
+        <is>
+          <t>Drei Forschungsartikel für „EU AI Act“</t>
+        </is>
+      </c>
+      <c r="C54" s="22" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="D54" s="22" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E54" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 30.10.2026</t>
+        </is>
+      </c>
+      <c r="F54" s="22" t="inlineStr">
+        <is>
+          <t>Zurückgezogen (verworfen); nichts geändert.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="22" t="inlineStr">
+        <is>
+          <t>REQ-54</t>
+        </is>
+      </c>
+      <c r="B55" s="22" t="inlineStr">
+        <is>
+          <t>Keine Möglichkeit, über das Interface neue Datenbanken anzulegen</t>
+        </is>
+      </c>
+      <c r="C55" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="D55" s="22" t="inlineStr">
+        <is>
+          <t>3.5.1</t>
+        </is>
+      </c>
+      <c r="E55" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 30.10.2026</t>
+        </is>
+      </c>
+      <c r="F55" s="22" t="inlineStr">
+        <is>
+          <t>„+ Add new data“ in der Datenbankleiste entfernt; Upload über Documents bleibt.</t>
         </is>
       </c>
     </row>
@@ -2437,7 +2501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -4063,7 +4127,7 @@
         </is>
       </c>
     </row>
-    <row r="32">
+    <row r="32" s="11">
       <c r="A32" s="22" t="inlineStr">
         <is>
           <t>REQ-52</t>
@@ -4112,6 +4176,110 @@
       <c r="J32" s="22" t="inlineStr">
         <is>
           <t>Frontend-Filter (PUBLIC_DBS, applyDbGate, dbGateFilter, dbScope); Feld „Password“ + „Lock“ im Header; Freischaltung in localStorage. Headless-Browser-Test bestanden. Hinweis: kein Zugriffsschutz – die API liefert weiterhin alle Datenbanken, das Passwort steht im Frontend-Code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" s="11">
+      <c r="A33" s="22" t="inlineStr">
+        <is>
+          <t>REQ-53</t>
+        </is>
+      </c>
+      <c r="B33" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C33" s="22" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D33" s="22" t="inlineStr">
+        <is>
+          <t>ergänze nun als scientific paper zuir datenbank eu ai act folgende paper [1-s2.0-S0160791X25002544-main.pdf, Laux et al. 2023 Regulation &amp; Governance, s41649-024-00304-6.pdf] · später: „Die 3 forschungsartikel von eben sollen doch nicht in eder eu ei act datenbank sein.“</t>
+        </is>
+      </c>
+      <c r="E33" s="22" t="inlineStr">
+        <is>
+          <t>Drei wissenschaftliche Artikel SOLLEN als Research papers der Datenbank „EU AI Act“ zugeordnet werden.</t>
+        </is>
+      </c>
+      <c r="F33" s="22" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G33" s="22" t="inlineStr">
+        <is>
+          <t>Daten</t>
+        </is>
+      </c>
+      <c r="H33" s="22" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="I33" s="22" t="inlineStr">
+        <is>
+          <t>Verworfen</t>
+        </is>
+      </c>
+      <c r="J33" s="22" t="inlineStr">
+        <is>
+          <t>Vom Anfragenden zurückgezogen. Vorbereitete Dateien (research/EUAIA/papers/), Summaries und Code-Änderungen wurden wieder entfernt; der erste Artikel liegt unverändert in LDK.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="22" t="inlineStr">
+        <is>
+          <t>REQ-54</t>
+        </is>
+      </c>
+      <c r="B34" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C34" s="22" t="inlineStr">
+        <is>
+          <t>3.5.1</t>
+        </is>
+      </c>
+      <c r="D34" s="22" t="inlineStr">
+        <is>
+          <t>entferne die möglichkeit neue datenbanken anlegen zu können über das interface</t>
+        </is>
+      </c>
+      <c r="E34" s="22" t="inlineStr">
+        <is>
+          <t>Das Interface DARF NICHT die Möglichkeit bieten, neue Datenbanken anzulegen; der Button „+ Add new data“ in der Datenbankleiste MUSS entfernt werden.</t>
+        </is>
+      </c>
+      <c r="F34" s="22" t="inlineStr">
+        <is>
+          <t>Datenbankleiste ohne „+ Add new data“; keine Stelle im Interface legt Datenbanken an; Hochladen in bestehende Datenbanken über Documents → + Upload funktioniert weiter.</t>
+        </is>
+      </c>
+      <c r="G34" s="22" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="H34" s="22" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="I34" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="J34" s="22" t="inlineStr">
+        <is>
+          <t>Button entfernt, Handbuch und Quick Reference angepasst. Headless-Browser-Test bestanden. Datenbanken waren schon vorher fest im Backend konfiguriert.</t>
         </is>
       </c>
     </row>
@@ -4139,7 +4307,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="130" customWidth="1" style="10" min="1" max="1"/>
@@ -4271,10 +4439,17 @@
         </is>
       </c>
     </row>
-    <row r="19">
+    <row r="19" s="11">
       <c r="A19" s="24" t="inlineStr">
         <is>
           <t>Release 3.5.0 (30.10.2026, Minor): REQ-52 (nur „EU AI Act“ ohne Passwort sichtbar; übrige Datenbanken nach Passwort neben dem OpenRouter-Key).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="24" t="inlineStr">
+        <is>
+          <t>Release 3.5.1 (30.10.2026, Patch): REQ-54 („+ Add new data“ aus der Datenbankleiste entfernt); REQ-53 (drei Paper für EU AI Act) zurückgezogen.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ALITA v3.6.0 – new database "Wachter" (REQ-55)
- Database WACHTER ("Wachter", shield icon, violet) in backend defaults,
  .env.example and front end (list, name, icon, colours, 3D view)
- research/WACHTER/papers (gitignored): Laux, Wachter & Mittelstadt 2024;
  Ho & Caals 2024, with curated summaries
- Hidden without the password like all databases except EU AI Act; tests 95 passed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiw6EWVWF8ScrYC2GD7
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -700,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -2438,7 +2438,7 @@
         </is>
       </c>
     </row>
-    <row r="55">
+    <row r="55" s="11">
       <c r="A55" s="22" t="inlineStr">
         <is>
           <t>REQ-54</t>
@@ -2467,6 +2467,38 @@
       <c r="F55" s="22" t="inlineStr">
         <is>
           <t>„+ Add new data“ in der Datenbankleiste entfernt; Upload über Documents bleibt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="22" t="inlineStr">
+        <is>
+          <t>REQ-55</t>
+        </is>
+      </c>
+      <c r="B56" s="22" t="inlineStr">
+        <is>
+          <t>Neue Datenbank „Wachter“ mit zwei Papern</t>
+        </is>
+      </c>
+      <c r="C56" s="22" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
+        </is>
+      </c>
+      <c r="D56" s="22" t="inlineStr">
+        <is>
+          <t>3.6.0</t>
+        </is>
+      </c>
+      <c r="E56" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 30.10.2026</t>
+        </is>
+      </c>
+      <c r="F56" s="22" t="inlineStr">
+        <is>
+          <t>ID WACHTER; Paper in research/WACHTER/papers/ mit kuratierten Summaries; Einlesen per Docker ausstehend.</t>
         </is>
       </c>
     </row>
@@ -2501,7 +2533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -4231,7 +4263,7 @@
         </is>
       </c>
     </row>
-    <row r="34">
+    <row r="34" s="11">
       <c r="A34" s="22" t="inlineStr">
         <is>
           <t>REQ-54</t>
@@ -4280,6 +4312,58 @@
       <c r="J34" s="22" t="inlineStr">
         <is>
           <t>Button entfernt, Handbuch und Quick Reference angepasst. Headless-Browser-Test bestanden. Datenbanken waren schon vorher fest im Backend konfiguriert.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="22" t="inlineStr">
+        <is>
+          <t>REQ-55</t>
+        </is>
+      </c>
+      <c r="B35" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C35" s="22" t="inlineStr">
+        <is>
+          <t>3.6.0</t>
+        </is>
+      </c>
+      <c r="D35" s="22" t="inlineStr">
+        <is>
+          <t>Mach eine neue datenbank mit diesen papern. nenn sie wachter [Laux et al. 2023/2024, Regulation &amp; Governance; s41649-024-00304-6.pdf]</t>
+        </is>
+      </c>
+      <c r="E35" s="22" t="inlineStr">
+        <is>
+          <t>Es MUSS eine neue Datenbank „Wachter“ geben, die die beiden Paper (Laux, Wachter &amp; Mittelstadt 2024; Ho &amp; Caals 2024) als Research papers enthält.</t>
+        </is>
+      </c>
+      <c r="F35" s="22" t="inlineStr">
+        <is>
+          <t>Datenbankleiste (mit Passwort) zeigt „Wachter“ mit eigenem Symbol und Farbe; nach „ingest all /research“ enthält Wachter 2 Paper mit kuratierter Summary, Titel, Autoren und Datum; Chat mit Auswahl Wachter findet Inhalte beider Paper.</t>
+        </is>
+      </c>
+      <c r="G35" s="22" t="inlineStr">
+        <is>
+          <t>Backend · Frontend · Daten</t>
+        </is>
+      </c>
+      <c r="H35" s="22" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="I35" s="22" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
+        </is>
+      </c>
+      <c r="J35" s="22" t="inlineStr">
+        <is>
+          <t>ID WACHTER in config.py, .env.example, databases.js, CSS; research/WACHTER/papers/ mit _summaries.yaml. Offline geprüft (DB-Zuordnung, Summaries), Tests 95 passed, Browser-Test der Datenbankleiste. Ohne Passwort ausgeblendet (REQ-52). Einlesen per Docker ausstehend.</t>
         </is>
       </c>
     </row>
@@ -4307,7 +4391,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="130" customWidth="1" style="10" min="1" max="1"/>
@@ -4446,10 +4530,17 @@
         </is>
       </c>
     </row>
-    <row r="20">
+    <row r="20" s="11">
       <c r="A20" s="24" t="inlineStr">
         <is>
           <t>Release 3.5.1 (30.10.2026, Patch): REQ-54 („+ Add new data“ aus der Datenbankleiste entfernt); REQ-53 (drei Paper für EU AI Act) zurückgezogen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="24" t="inlineStr">
+        <is>
+          <t>Release 3.6.0 (30.10.2026, Minor): REQ-55 (neue Datenbank „Wachter“ mit zwei Papern zu vertrauenswürdiger KI und AI Act).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ALITA v3.6.1 – Wachter visible without the password (REQ-56)
- PUBLIC_DBS = EU AI Act + Wachter; empty selection searches both
- Tooltips, user manual and Wachter README updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiw6EWVWF8ScrYC2GD7
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -700,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -2470,7 +2470,7 @@
         </is>
       </c>
     </row>
-    <row r="56">
+    <row r="56" s="11">
       <c r="A56" s="22" t="inlineStr">
         <is>
           <t>REQ-55</t>
@@ -2499,6 +2499,38 @@
       <c r="F56" s="22" t="inlineStr">
         <is>
           <t>ID WACHTER; Paper in research/WACHTER/papers/ mit kuratierten Summaries; Einlesen per Docker ausstehend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="22" t="inlineStr">
+        <is>
+          <t>REQ-56</t>
+        </is>
+      </c>
+      <c r="B57" s="22" t="inlineStr">
+        <is>
+          <t>Wachter ohne Passwort sichtbar wie EU AI Act</t>
+        </is>
+      </c>
+      <c r="C57" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="D57" s="22" t="inlineStr">
+        <is>
+          <t>3.6.1</t>
+        </is>
+      </c>
+      <c r="E57" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 30.10.2026</t>
+        </is>
+      </c>
+      <c r="F57" s="22" t="inlineStr">
+        <is>
+          <t>PUBLIC_DBS = EUAIA, WACHTER.</t>
         </is>
       </c>
     </row>
@@ -2533,7 +2565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J35"/>
+  <dimension ref="A1:J36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -4315,7 +4347,7 @@
         </is>
       </c>
     </row>
-    <row r="35">
+    <row r="35" s="11">
       <c r="A35" s="22" t="inlineStr">
         <is>
           <t>REQ-55</t>
@@ -4364,6 +4396,58 @@
       <c r="J35" s="22" t="inlineStr">
         <is>
           <t>ID WACHTER in config.py, .env.example, databases.js, CSS; research/WACHTER/papers/ mit _summaries.yaml. Offline geprüft (DB-Zuordnung, Summaries), Tests 95 passed, Browser-Test der Datenbankleiste. Ohne Passwort ausgeblendet (REQ-52). Einlesen per Docker ausstehend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="22" t="inlineStr">
+        <is>
+          <t>REQ-56</t>
+        </is>
+      </c>
+      <c r="B36" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C36" s="22" t="inlineStr">
+        <is>
+          <t>3.6.1</t>
+        </is>
+      </c>
+      <c r="D36" s="22" t="inlineStr">
+        <is>
+          <t>wachter soll auch defaukt sichtbar sein wie e aia ct</t>
+        </is>
+      </c>
+      <c r="E36" s="22" t="inlineStr">
+        <is>
+          <t>Die Datenbank „Wachter“ MUSS wie „EU AI Act“ ohne Passwort sichtbar sein.</t>
+        </is>
+      </c>
+      <c r="F36" s="22" t="inlineStr">
+        <is>
+          <t>Ohne Passwort zeigt die Datenbankleiste EU AI Act und Wachter; leere Auswahl sucht in beiden; mit Passwort alle Datenbanken.</t>
+        </is>
+      </c>
+      <c r="G36" s="22" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="H36" s="22" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="I36" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="J36" s="22" t="inlineStr">
+        <is>
+          <t>PUBLIC_DBS um WACHTER ergänzt; Tooltips und Handbuch angepasst. Headless-Browser-Test bestanden.</t>
         </is>
       </c>
     </row>
@@ -4391,7 +4475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="130" customWidth="1" style="10" min="1" max="1"/>
@@ -4537,10 +4621,17 @@
         </is>
       </c>
     </row>
-    <row r="21">
+    <row r="21" s="11">
       <c r="A21" s="24" t="inlineStr">
         <is>
           <t>Release 3.6.0 (30.10.2026, Minor): REQ-55 (neue Datenbank „Wachter“ mit zwei Papern zu vertrauenswürdiger KI und AI Act).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="24" t="inlineStr">
+        <is>
+          <t>Release 3.6.1 (30.10.2026, Patch): REQ-56 (Wachter wie EU AI Act ohne Passwort sichtbar).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ALITA v3.6.2 – documentation tabs behind the password (REQ-57)
- "ISO 42001/EUAIACT Docs" and "Technical Documentation" hidden while the
  database password is not entered (LOCKED_PAGES); #compliance/#tech open B
- Lock leaves a hidden tab; tests 183 passed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiw6EWVWF8ScrYC2GD7
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -700,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -2502,7 +2502,7 @@
         </is>
       </c>
     </row>
-    <row r="57">
+    <row r="57" s="11">
       <c r="A57" s="22" t="inlineStr">
         <is>
           <t>REQ-56</t>
@@ -2531,6 +2531,38 @@
       <c r="F57" s="22" t="inlineStr">
         <is>
           <t>PUBLIC_DBS = EUAIA, WACHTER.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="22" t="inlineStr">
+        <is>
+          <t>REQ-57</t>
+        </is>
+      </c>
+      <c r="B58" s="22" t="inlineStr">
+        <is>
+          <t>Reiter „ISO 42001/EUAIACT Docs“ und „Technical Documentation“ ohne Passwort ausblenden</t>
+        </is>
+      </c>
+      <c r="C58" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="D58" s="22" t="inlineStr">
+        <is>
+          <t>3.6.2</t>
+        </is>
+      </c>
+      <c r="E58" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 31.10.2026</t>
+        </is>
+      </c>
+      <c r="F58" s="22" t="inlineStr">
+        <is>
+          <t>Wie die Datenbanken hinter dem Passwort (LOCKED_PAGES).</t>
         </is>
       </c>
     </row>
@@ -2565,7 +2597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J36"/>
+  <dimension ref="A1:J37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -4399,7 +4431,7 @@
         </is>
       </c>
     </row>
-    <row r="36">
+    <row r="36" s="11">
       <c r="A36" s="22" t="inlineStr">
         <is>
           <t>REQ-56</t>
@@ -4448,6 +4480,58 @@
       <c r="J36" s="22" t="inlineStr">
         <is>
           <t>PUBLIC_DBS um WACHTER ergänzt; Tooltips und Handbuch angepasst. Headless-Browser-Test bestanden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="22" t="inlineStr">
+        <is>
+          <t>REQ-57</t>
+        </is>
+      </c>
+      <c r="B37" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="C37" s="22" t="inlineStr">
+        <is>
+          <t>3.6.2</t>
+        </is>
+      </c>
+      <c r="D37" s="22" t="inlineStr">
+        <is>
+          <t>Hide  the menues "ISO 42001/EU AI Act Docs" and "Technical Documentation" as well</t>
+        </is>
+      </c>
+      <c r="E37" s="22" t="inlineStr">
+        <is>
+          <t>Die Reiter „ISO 42001/EUAIACT Docs“ und „Technical Documentation“ DÜRFEN ohne Passwort NICHT angezeigt werden; mit Passwort MÜSSEN sie wie bisher erscheinen.</t>
+        </is>
+      </c>
+      <c r="F37" s="22" t="inlineStr">
+        <is>
+          <t>Ohne Passwort: vier Reiter (B, A/B, Documents, Release Notes); Links #compliance/#tech öffnen B. Mit Passwort: sechs Reiter. „Lock“ blendet beide wieder aus und verlässt einen geöffneten Doku-Reiter.</t>
+        </is>
+      </c>
+      <c r="G37" s="22" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="H37" s="22" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="I37" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="J37" s="22" t="inlineStr">
+        <is>
+          <t>LOCKED_PAGES in databases.js, Umleitung in showPage, Lock-Pfad in setDbUnlocked. Headless-Browser-Test bestanden. Nur Anzeige: die Doku-APIs antworten weiter.</t>
         </is>
       </c>
     </row>
@@ -4475,7 +4559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="130" customWidth="1" style="10" min="1" max="1"/>
@@ -4628,10 +4712,17 @@
         </is>
       </c>
     </row>
-    <row r="22">
+    <row r="22" s="11">
       <c r="A22" s="24" t="inlineStr">
         <is>
           <t>Release 3.6.1 (30.10.2026, Patch): REQ-56 (Wachter wie EU AI Act ohne Passwort sichtbar).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="24" t="inlineStr">
+        <is>
+          <t>Release 3.6.2 (31.10.2026, Patch): REQ-57 (Doku-Reiter ISO 42001/EUAIACT und Technical Documentation ohne Passwort ausgeblendet).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ALITA v3.6.3 – release notes behind the password (REQ-58)
- "Release Notes" added to LOCKED_PAGES; the version number is plain text
  while locked; #release / #release-notes open B
- Tests 183 passed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiw6EWVWF8ScrYC2GD7
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -700,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F58"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -2534,7 +2534,7 @@
         </is>
       </c>
     </row>
-    <row r="58">
+    <row r="58" s="11">
       <c r="A58" s="22" t="inlineStr">
         <is>
           <t>REQ-57</t>
@@ -2563,6 +2563,38 @@
       <c r="F58" s="22" t="inlineStr">
         <is>
           <t>Wie die Datenbanken hinter dem Passwort (LOCKED_PAGES).</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="22" t="inlineStr">
+        <is>
+          <t>REQ-58</t>
+        </is>
+      </c>
+      <c r="B59" s="22" t="inlineStr">
+        <is>
+          <t>Reiter „Release Notes“ ohne Passwort ausblenden</t>
+        </is>
+      </c>
+      <c r="C59" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="D59" s="22" t="inlineStr">
+        <is>
+          <t>3.6.3</t>
+        </is>
+      </c>
+      <c r="E59" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 31.10.2026</t>
+        </is>
+      </c>
+      <c r="F59" s="22" t="inlineStr">
+        <is>
+          <t>Wie die Doku-Reiter hinter dem Passwort (LOCKED_PAGES).</t>
         </is>
       </c>
     </row>
@@ -2597,7 +2629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -4483,7 +4515,7 @@
         </is>
       </c>
     </row>
-    <row r="37">
+    <row r="37" s="11">
       <c r="A37" s="22" t="inlineStr">
         <is>
           <t>REQ-57</t>
@@ -4532,6 +4564,58 @@
       <c r="J37" s="22" t="inlineStr">
         <is>
           <t>LOCKED_PAGES in databases.js, Umleitung in showPage, Lock-Pfad in setDbUnlocked. Headless-Browser-Test bestanden. Nur Anzeige: die Doku-APIs antworten weiter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="22" t="inlineStr">
+        <is>
+          <t>REQ-58</t>
+        </is>
+      </c>
+      <c r="B38" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="C38" s="22" t="inlineStr">
+        <is>
+          <t>3.6.3</t>
+        </is>
+      </c>
+      <c r="D38" s="22" t="inlineStr">
+        <is>
+          <t>hide release notes as wel</t>
+        </is>
+      </c>
+      <c r="E38" s="22" t="inlineStr">
+        <is>
+          <t>Der Reiter „Release Notes“ DARF ohne Passwort NICHT angezeigt werden; mit Passwort MUSS er wie bisher erscheinen.</t>
+        </is>
+      </c>
+      <c r="F38" s="22" t="inlineStr">
+        <is>
+          <t>Ohne Passwort: drei Reiter (B, A/B, Documents), Versionsnummer öffnet keine Release Notes, #release-notes öffnet B. Mit Passwort: sechs Reiter, Versionsnummer öffnet die Release Notes.</t>
+        </is>
+      </c>
+      <c r="G38" s="22" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="H38" s="22" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="I38" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="J38" s="22" t="inlineStr">
+        <is>
+          <t>„release“ in LOCKED_PAGES; Versions-Button ohne Passwort deaktiviert. Headless-Browser-Test bestanden. Nur Anzeige: /api/release-notes antwortet weiter.</t>
         </is>
       </c>
     </row>
@@ -4559,7 +4643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="130" customWidth="1" style="10" min="1" max="1"/>
@@ -4719,10 +4803,17 @@
         </is>
       </c>
     </row>
-    <row r="23">
+    <row r="23" s="11">
       <c r="A23" s="24" t="inlineStr">
         <is>
           <t>Release 3.6.2 (31.10.2026, Patch): REQ-57 (Doku-Reiter ISO 42001/EUAIACT und Technical Documentation ohne Passwort ausgeblendet).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="24" t="inlineStr">
+        <is>
+          <t>Release 3.6.3 (31.10.2026, Patch): REQ-58 (Release Notes ohne Passwort ausgeblendet).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ALITA v3.7.0 – compare the clusters of two databases; Graph Chat across databases (REQ-59 – REQ-61)
- GET /api/clusters/relations: cross-database cluster relations (centroid
  similarity of summary vectors, bridging documents) – cluster_relations.py
- B page: dropdown "Compare" (EU AI Act <-> Wachter first), violet dashed
  relation lines in 2D and 3D, side panel with Select/Ask – cluster-compare.js
- Graph Chat: clusters from several databases are searched per database and
  interleaved; the prompt gets their relations; answer shows the scope
- REQ-60: the standard added in 3.3.1 removed from code, tests, docs, release
  notes and requirements log; new `ingest delete --norm ID`
- REQ-61: staged refactoring plan (docs/technical/architecture), stage 0
- Tests 188 passed; ruff clean; data.js regenerated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiw6EWVWF8ScrYC2GD7
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -700,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F62"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -2286,12 +2286,12 @@
       </c>
       <c r="B50" s="22" t="inlineStr">
         <is>
-          <t>Erster Standard: DIN SPEC 92005:2024-03 (Uncertainty quantification in machine learning)</t>
+          <t>Erster Standard für „EU AI Act“ (in 3.7.0 wieder entfernt)</t>
         </is>
       </c>
       <c r="C50" s="22" t="inlineStr">
         <is>
-          <t>In Arbeit</t>
+          <t>Erledigt (erklärt)</t>
         </is>
       </c>
       <c r="D50" s="22" t="inlineStr">
@@ -2306,7 +2306,7 @@
       </c>
       <c r="F50" s="22" t="inlineStr">
         <is>
-          <t>Datei und _legal.yaml in research/EUAIA/standards/ (published, ab 1.3.2024). Personalisierte Lizenzstempel (Name, Kundennummer, Download-ID, Zeit) werden beim Auslesen jeder PDF entfernt. Normen: Begriffe als eigene Bestandteile (28), Anhangstatus, Anhang-Gliederung C.1.2.1, Tabellenzeilen in Anhängen als Text. Offline geprüft: kein Stempel, Abschnitte 1–7, 28 Begriffe, Anhänge A–C, 174 Text Units. Lizenz vor dem Einlesen prüfen (Einzelplatzlizenz, externer KI-Dienst).</t>
+          <t>Parser für Standards (Begriffe, Anhangstatus, Anhang-Gliederung) und das Entfernen von Lizenzstempeln aus PDFs bleiben; der Standard selbst und alle Verweise darauf wurden in 3.7.0 entfernt (REQ-60).</t>
         </is>
       </c>
     </row>
@@ -2338,7 +2338,7 @@
       </c>
       <c r="F51" s="22" t="inlineStr">
         <is>
-          <t>Zweiter Eintrag in research/EUAIA/standards/_legal.yaml (published, Juni 2026; frei verfügbar). Parser: „Appendix A.“ als Anhang, „References“/„Bibliography“ als eigene Anlage. Offline geprüft: Abschnitte 1–4.7, References, Anhänge A–D. Erster Upload war versehentlich nochmals die DIN SPEC 92005 (byte-identisch) – dafür nichts geändert. Einlesen per Docker steht aus.</t>
+          <t>Zweiter Eintrag in research/EUAIA/standards/_legal.yaml (published, Juni 2026; frei verfügbar). Parser: „Appendix A.“ als Anhang, „References“/„Bibliography“ als eigene Anlage. Offline geprüft: Abschnitte 1–4.7, References, Anhänge A–D. Einlesen per Docker steht aus.</t>
         </is>
       </c>
     </row>
@@ -2566,7 +2566,7 @@
         </is>
       </c>
     </row>
-    <row r="59">
+    <row r="59" s="11">
       <c r="A59" s="22" t="inlineStr">
         <is>
           <t>REQ-58</t>
@@ -2595,6 +2595,102 @@
       <c r="F59" s="22" t="inlineStr">
         <is>
           <t>Wie die Doku-Reiter hinter dem Passwort (LOCKED_PAGES).</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" s="11">
+      <c r="A60" s="22" t="inlineStr">
+        <is>
+          <t>REQ-59</t>
+        </is>
+      </c>
+      <c r="B60" s="22" t="inlineStr">
+        <is>
+          <t>Cluster zweier Datenbanken vergleichen (Dropdown, Linien in der Karte), Graph Chat über Datenbanken hinweg in den Clustern</t>
+        </is>
+      </c>
+      <c r="C60" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="D60" s="22" t="inlineStr">
+        <is>
+          <t>3.7.0</t>
+        </is>
+      </c>
+      <c r="E60" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 31.10.2026</t>
+        </is>
+      </c>
+      <c r="F60" s="22" t="inlineStr">
+        <is>
+          <t>Dropdown „Compare“, /api/clusters/relations, Graph Chat je Datenbank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" s="11">
+      <c r="A61" s="22" t="inlineStr">
+        <is>
+          <t>REQ-60</t>
+        </is>
+      </c>
+      <c r="B61" s="22" t="inlineStr">
+        <is>
+          <t>Standard aus 3.3.1 vollständig entfernen</t>
+        </is>
+      </c>
+      <c r="C61" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="D61" s="22" t="inlineStr">
+        <is>
+          <t>3.7.0</t>
+        </is>
+      </c>
+      <c r="E61" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 31.10.2026</t>
+        </is>
+      </c>
+      <c r="F61" s="22" t="inlineStr">
+        <is>
+          <t>Überall entfernt; Neo4j/Modellablage mit ingest delete --norm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="22" t="inlineStr">
+        <is>
+          <t>REQ-61</t>
+        </is>
+      </c>
+      <c r="B62" s="22" t="inlineStr">
+        <is>
+          <t>Codebasis schrittweise refaktorieren</t>
+        </is>
+      </c>
+      <c r="C62" s="22" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
+        </is>
+      </c>
+      <c r="D62" s="22" t="inlineStr">
+        <is>
+          <t>3.7.0 –</t>
+        </is>
+      </c>
+      <c r="E62" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 31.10.2026</t>
+        </is>
+      </c>
+      <c r="F62" s="22" t="inlineStr">
+        <is>
+          <t>Stufe 0 erledigt; Plan in docs/technical/architecture.</t>
         </is>
       </c>
     </row>
@@ -2629,7 +2725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -4117,17 +4213,17 @@
       </c>
       <c r="D29" s="22" t="inlineStr">
         <is>
-          <t>jetzt ein standard [3521675.PDF – DIN SPEC 92005:2024-03]</t>
+          <t>jetzt ein standard [Datei – in 3.7.0 entfernt]</t>
         </is>
       </c>
       <c r="E29" s="22" t="inlineStr">
         <is>
-          <t>Die DIN SPEC 92005:2024-03 MUSS als Standard in „EU AI Act“ geführt werden, gegliedert in Abschnitte, Begriffe und Anhänge. Personenbezogene Lizenzstempel des Downloads DÜRFEN NICHT in Index, Graph oder Prompts gelangen.</t>
+          <t>Ein erster Standard MUSS in „EU AI Act“ geführt werden, gegliedert in Abschnitte, Begriffe und Anhänge. Personenbezogene Lizenzstempel des Downloads DÜRFEN NICHT in Index, Graph oder Prompts gelangen.</t>
         </is>
       </c>
       <c r="F29" s="22" t="inlineStr">
         <is>
-          <t>Nach „ingest standard /research/EUAIA/standards“: Standard „DIN SPEC 92005“ (▲) in EU AI Act; 28 Begriffe (z. B. „uncertainty quantification“), Anhänge A–C; kein Name/keine Kundennummer im Text; Frage „How does DIN SPEC 92005 define aleatoric uncertainty?“ nennt Clause 3.3.</t>
+          <t>Standard gegliedert in Abschnitte, Begriffe und Anhänge; kein Name/keine Kundennummer im Text.</t>
         </is>
       </c>
       <c r="G29" s="22" t="inlineStr">
@@ -4142,12 +4238,12 @@
       </c>
       <c r="I29" s="22" t="inlineStr">
         <is>
-          <t>In Arbeit</t>
+          <t>Verworfen</t>
         </is>
       </c>
       <c r="J29" s="22" t="inlineStr">
         <is>
-          <t>Tests 93 passed; ingest_legal als standard mit Platzhaltern durchgelaufen (92 Bestandteile). Offen: Lizenz der DIN-Media-Datei für gemeinsame Instanz und externen KI-Dienst prüfen; danach Einlesen per Docker.</t>
+          <t>Parser und Entfernen der Lizenzstempel umgesetzt (Tests 93 passed). Der Standard selbst wurde in 3.7.0 auf Wunsch vollständig entfernt (REQ-60).</t>
         </is>
       </c>
     </row>
@@ -4169,7 +4265,7 @@
       </c>
       <c r="D30" s="22" t="inlineStr">
         <is>
-          <t>nochmal so ein e art standard [3521675.PDF – identisch mit DIN SPEC 92005] / [NIST.SP.800-18r2.pdf]</t>
+          <t>nochmal so ein e art standard [Datei 1 – identisch mit dem ersten Standard, entfernt] / [NIST.SP.800-18r2.pdf]</t>
         </is>
       </c>
       <c r="E30" s="22" t="inlineStr">
@@ -4179,7 +4275,7 @@
       </c>
       <c r="F30" s="22" t="inlineStr">
         <is>
-          <t>Nach „ingest standard /research/EUAIA/standards“: zwei Standards (DIN SPEC 92005, NIST SP 800-18r2); NIST mit 28 Abschnitten, References und Anhängen A–D; Frage „What does NIST SP 800-18r2 say about consolidated system plans?“ nennt Clause 2.4.</t>
+          <t>Nach „ingest standard /research/EUAIA/standards“: Standard NIST SP 800-18r2 mit 28 Abschnitten, References und Anhängen A–D; Frage „What does NIST SP 800-18r2 say about consolidated system plans?“ nennt Clause 2.4.</t>
         </is>
       </c>
       <c r="G30" s="22" t="inlineStr">
@@ -4199,7 +4295,7 @@
       </c>
       <c r="J30" s="22" t="inlineStr">
         <is>
-          <t>Tests 94 passed; ingest_legal für beide Standards mit Platzhaltern durchgelaufen. Einlesen per Docker mit -e OPENROUTER_API_KEY steht aus (DIN-Lizenz vorher prüfen).</t>
+          <t>Tests 94 passed; ingest_legal für den Standard mit Platzhaltern durchgelaufen.</t>
         </is>
       </c>
     </row>
@@ -4567,7 +4663,7 @@
         </is>
       </c>
     </row>
-    <row r="38">
+    <row r="38" s="11">
       <c r="A38" s="22" t="inlineStr">
         <is>
           <t>REQ-58</t>
@@ -4616,6 +4712,162 @@
       <c r="J38" s="22" t="inlineStr">
         <is>
           <t>„release“ in LOCKED_PAGES; Versions-Button ohne Passwort deaktiviert. Headless-Browser-Test bestanden. Nur Anzeige: /api/release-notes antwortet weiter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" s="11">
+      <c r="A39" s="22" t="inlineStr">
+        <is>
+          <t>REQ-59</t>
+        </is>
+      </c>
+      <c r="B39" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="C39" s="22" t="inlineStr">
+        <is>
+          <t>3.7.0</t>
+        </is>
+      </c>
+      <c r="D39" s="22" t="inlineStr">
+        <is>
+          <t>Make cluster analysis for eu ai act and wachter database together. I want to selecte from a drop down that I want to compare these 2 datgabases cluster. then these cluster relations are also decpited on the image that is already there. Please completely remove [the standard] from everywhere. then after that refactor the whole code basis. The goal is that I can use the chat graph to requery inside the clusters across databsaes</t>
+        </is>
+      </c>
+      <c r="E39" s="22" t="inlineStr">
+        <is>
+          <t>Die Cluster von „EU AI Act“ und „Wachter“ MÜSSEN gemeinsam analysiert werden können: über ein Dropdown wird ein Datenbankpaar zum Vergleich gewählt; die Beziehungen zwischen den Clustern beider Datenbanken MÜSSEN in der bestehenden Wissenskarte dargestellt werden. Der Graph Chat MUSS in den ausgewählten Clustern über Datenbankgrenzen hinweg erneut suchen können.</t>
+        </is>
+      </c>
+      <c r="F39" s="22" t="inlineStr">
+        <is>
+          <t>Dropdown „Compare“ zeigt „EU AI Act ↔ Wachter“; nach Auswahl violette gestrichelte Linien mit Ähnlichkeit zwischen Clustern beider Datenbanken (2D und 3D); „Select“/„Ask“ bzw. Klick auf eine Linie wählt beide Cluster; Graph-Chat-Anfrage enthält beide Datenbanken und beide Cluster, Treffer aus beiden Datenbanken.</t>
+        </is>
+      </c>
+      <c r="G39" s="22" t="inlineStr">
+        <is>
+          <t>Backend · Frontend · Graph Chat</t>
+        </is>
+      </c>
+      <c r="H39" s="22" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="I39" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="J39" s="22" t="inlineStr">
+        <is>
+          <t>/api/clusters/relations (Zentroid-Ähnlichkeit, Brücken), cluster_relations.py, cluster-compare.js, Graph Chat retrieve_across (je Datenbank suchen, abwechselnd zusammenführen) + Beziehungen im Prompt. Live: C6 ↔ C8 0,76; C7 ↔ C8 0,33. Tests 188 passed; Headless-Browser-Test bestanden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" s="11">
+      <c r="A40" s="22" t="inlineStr">
+        <is>
+          <t>REQ-60</t>
+        </is>
+      </c>
+      <c r="B40" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="C40" s="22" t="inlineStr">
+        <is>
+          <t>3.7.0</t>
+        </is>
+      </c>
+      <c r="D40" s="22" t="inlineStr">
+        <is>
+          <t>Make cluster analysis for eu ai act and wachter database together. I want to selecte from a drop down that I want to compare these 2 datgabases cluster. then these cluster relations are also decpited on the image that is already there. Please completely remove [the standard] from everywhere. then after that refactor the whole code basis. The goal is that I can use the chat graph to requery inside the clusters across databsaes</t>
+        </is>
+      </c>
+      <c r="E40" s="22" t="inlineStr">
+        <is>
+          <t>Der in 3.3.1 aufgenommene Standard DARF an keiner Stelle mehr vorkommen: nicht im Datenordner, nicht im Index (Qdrant, Graph, Modellablage), nicht in Code, Tests, Dokumentation, Release Notes und Anforderungsprotokoll.</t>
+        </is>
+      </c>
+      <c r="F40" s="22" t="inlineStr">
+        <is>
+          <t>Suche nach Name/Nummer des Standards im Repository, im Datenordner und im lokalen Index ohne Treffer; die Parser-Funktionen und das Entfernen von Lizenzstempeln bleiben.</t>
+        </is>
+      </c>
+      <c r="G40" s="22" t="inlineStr">
+        <is>
+          <t>Daten · Backend · Doku</t>
+        </is>
+      </c>
+      <c r="H40" s="22" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="I40" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="J40" s="22" t="inlineStr">
+        <is>
+          <t>Datei und _legal.yaml-Eintrag gelöscht; Erwähnungen entfernt (CHANGELOG, README, Status, Log, Testdaten, Kommentare); 141 Stellen + Dokument aus Qdrant gelöscht, veraltete Clustertexte geleert; neues Kommando ingest delete --norm für Neo4j und Modellablage. Exporte im Download-Ordner bereinigt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="22" t="inlineStr">
+        <is>
+          <t>REQ-61</t>
+        </is>
+      </c>
+      <c r="B41" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="C41" s="22" t="inlineStr">
+        <is>
+          <t>3.7.0 –</t>
+        </is>
+      </c>
+      <c r="D41" s="22" t="inlineStr">
+        <is>
+          <t>Make cluster analysis for eu ai act and wachter database together. I want to selecte from a drop down that I want to compare these 2 datgabases cluster. then these cluster relations are also decpited on the image that is already there. Please completely remove [the standard] from everywhere. then after that refactor the whole code basis. The goal is that I can use the chat graph to requery inside the clusters across databsaes</t>
+        </is>
+      </c>
+      <c r="E41" s="22" t="inlineStr">
+        <is>
+          <t>Die Codebasis SOLL schrittweise (mehrere PRs) refaktoriert werden, mit dem Ziel, dass der Graph Chat innerhalb von Clustern über Datenbanken hinweg erneut suchen kann; das Verhalten DARF sich je Stufe nicht ungewollt ändern.</t>
+        </is>
+      </c>
+      <c r="F41" s="22" t="inlineStr">
+        <is>
+          <t>Plan mit Stufen in docs/technical/architecture/01-refactoring-plan.md; jede Stufe ein PR mit grüner CI und unveränderten Tests.</t>
+        </is>
+      </c>
+      <c r="G41" s="22" t="inlineStr">
+        <is>
+          <t>Architektur</t>
+        </is>
+      </c>
+      <c r="H41" s="22" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="I41" s="22" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
+        </is>
+      </c>
+      <c r="J41" s="22" t="inlineStr">
+        <is>
+          <t>Stufe 0 in 3.7.0 (eigene Module für den Datenbankvergleich); Stufen 1–5 folgen.</t>
         </is>
       </c>
     </row>
@@ -4643,7 +4895,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="130" customWidth="1" style="10" min="1" max="1"/>
@@ -4757,7 +5009,7 @@
     <row r="16">
       <c r="A16" s="24" t="inlineStr">
         <is>
-          <t>Release 3.3.1 (30.10.2026, Patch): REQ-49 (DIN SPEC 92005 als erster Standard, Lizenzstempel werden entfernt) vorbereitet und offline geprüft; Lizenz prüfen, dann Einlesen per Docker. Release Notes: CHANGELOG.md, Abschnitt [3.3.1].</t>
+          <t>Release 3.3.1 (30.10.2026, Patch): REQ-49 (Lizenzstempel werden aus PDFs entfernt; Parser für Standards). Release Notes: CHANGELOG.md, Abschnitt [3.3.1].</t>
         </is>
       </c>
     </row>
@@ -4810,10 +5062,17 @@
         </is>
       </c>
     </row>
-    <row r="24">
+    <row r="24" s="11">
       <c r="A24" s="24" t="inlineStr">
         <is>
           <t>Release 3.6.3 (31.10.2026, Patch): REQ-58 (Release Notes ohne Passwort ausgeblendet).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="24" t="inlineStr">
+        <is>
+          <t>Release 3.7.0 (31.10.2026, Minor): REQ-59 (Cluster zweier Datenbanken vergleichen, Graph Chat über Datenbanken), REQ-60 (Standard aus 3.3.1 vollständig entfernt), REQ-61 (Refactoring, Stufe 0).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ALITA v3.7.1 – B page: database bar, window to the outside and B explainer in one row (REQ-62)
- Three boxes side by side (.bar-row); #bTop only on the B page; the knowledge
  map moves up; below 980 px the boxes wrap

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiw6EWVWF8ScrYC2GD7
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -700,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F62"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -2662,7 +2662,7 @@
         </is>
       </c>
     </row>
-    <row r="62">
+    <row r="62" s="11">
       <c r="A62" s="22" t="inlineStr">
         <is>
           <t>REQ-61</t>
@@ -2691,6 +2691,38 @@
       <c r="F62" s="22" t="inlineStr">
         <is>
           <t>Stufe 0 erledigt; Plan in docs/technical/architecture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="22" t="inlineStr">
+        <is>
+          <t>REQ-62</t>
+        </is>
+      </c>
+      <c r="B63" s="22" t="inlineStr">
+        <is>
+          <t>B-Seite: Datenbankleiste, „Window to the outside“ und B-Erklärung als drei Kästen nebeneinander</t>
+        </is>
+      </c>
+      <c r="C63" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="D63" s="22" t="inlineStr">
+        <is>
+          <t>3.7.1</t>
+        </is>
+      </c>
+      <c r="E63" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 31.10.2026</t>
+        </is>
+      </c>
+      <c r="F63" s="22" t="inlineStr">
+        <is>
+          <t>.bar-row, #bTop nur auf B.</t>
         </is>
       </c>
     </row>
@@ -2725,7 +2757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -4819,7 +4851,7 @@
         </is>
       </c>
     </row>
-    <row r="41">
+    <row r="41" s="11">
       <c r="A41" s="22" t="inlineStr">
         <is>
           <t>REQ-61</t>
@@ -4868,6 +4900,58 @@
       <c r="J41" s="22" t="inlineStr">
         <is>
           <t>Stufe 0 in 3.7.0 (eigene Module für den Datenbankvergleich); Stufen 1–5 folgen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="22" t="inlineStr">
+        <is>
+          <t>REQ-62</t>
+        </is>
+      </c>
+      <c r="B42" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="C42" s="22" t="inlineStr">
+        <is>
+          <t>3.7.1</t>
+        </is>
+      </c>
+      <c r="D42" s="22" t="inlineStr">
+        <is>
+          <t>[Screenshot: „Window to the outside“ und B-Erklärung eingekreist, Pfeile in die freie Fläche der Datenbankleiste] · „it should be three own boxes not two boxes witrhin a box“</t>
+        </is>
+      </c>
+      <c r="E42" s="22" t="inlineStr">
+        <is>
+          <t>Auf der B-Seite MÜSSEN „Window to the outside“ und die B-Erklärung neben der Datenbankleiste stehen – als drei eigene Kästen in einer Zeile, nicht als Kästen innerhalb der Datenbankleiste.</t>
+        </is>
+      </c>
+      <c r="F42" s="22" t="inlineStr">
+        <is>
+          <t>B-Seite: Datenbankleiste, „Window to the outside“, B-Erklärung als drei Kästen nebeneinander; keine eigene Zeile darunter; andere Seiten: nur die Datenbankleiste in voller Breite; Pop-up öffnet weiter.</t>
+        </is>
+      </c>
+      <c r="G42" s="22" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="H42" s="22" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="I42" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="J42" s="22" t="inlineStr">
+        <is>
+          <t>.bar-row in index.html/tiles.css, #bTop nur auf B (showPage). Erster Entwurf (in der Leiste) auf Rückmeldung zu drei eigenen Kästen geändert. Lokal und headless geprüft.</t>
         </is>
       </c>
     </row>
@@ -4895,7 +4979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="130" customWidth="1" style="10" min="1" max="1"/>
@@ -5069,10 +5153,17 @@
         </is>
       </c>
     </row>
-    <row r="25">
+    <row r="25" s="11">
       <c r="A25" s="24" t="inlineStr">
         <is>
           <t>Release 3.7.0 (31.10.2026, Minor): REQ-59 (Cluster zweier Datenbanken vergleichen, Graph Chat über Datenbanken), REQ-60 (Standard aus 3.3.1 vollständig entfernt), REQ-61 (Refactoring, Stufe 0).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="24" t="inlineStr">
+        <is>
+          <t>Release 3.7.1 (31.10.2026, Patch): REQ-62 (drei Kästen in einer Zeile auf der B-Seite).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ALITA v3.7.2 – B page in three columns; Enlarge opens the map in its own window (REQ-63)
- Knowledge map | Projects & clusters | Graph Chat side by side
- map-window.js: '⤢ Enlarge' opens ?view=map (map only) in a separate browser
  window; cluster and database selection synced over a BroadcastChannel;
  overlay as fallback when pop-ups are blocked

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiw6EWVWF8ScrYC2GD7
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -700,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F63"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -2694,7 +2694,7 @@
         </is>
       </c>
     </row>
-    <row r="63">
+    <row r="63" s="11">
       <c r="A63" s="22" t="inlineStr">
         <is>
           <t>REQ-62</t>
@@ -2723,6 +2723,38 @@
       <c r="F63" s="22" t="inlineStr">
         <is>
           <t>.bar-row, #bTop nur auf B.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="22" t="inlineStr">
+        <is>
+          <t>REQ-63</t>
+        </is>
+      </c>
+      <c r="B64" s="22" t="inlineStr">
+        <is>
+          <t>B-Seite in drei Spalten; „Enlarge“ öffnet eigenes Fenster</t>
+        </is>
+      </c>
+      <c r="C64" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="D64" s="22" t="inlineStr">
+        <is>
+          <t>3.7.2</t>
+        </is>
+      </c>
+      <c r="E64" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 31.10.2026</t>
+        </is>
+      </c>
+      <c r="F64" s="22" t="inlineStr">
+        <is>
+          <t>Grid map|cluster|chat; map-window.js.</t>
         </is>
       </c>
     </row>
@@ -2757,7 +2789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J42"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -4903,7 +4935,7 @@
         </is>
       </c>
     </row>
-    <row r="42">
+    <row r="42" s="11">
       <c r="A42" s="22" t="inlineStr">
         <is>
           <t>REQ-62</t>
@@ -4952,6 +4984,58 @@
       <c r="J42" s="22" t="inlineStr">
         <is>
           <t>.bar-row in index.html/tiles.css, #bTop nur auf B (showPage). Erster Entwurf (in der Leiste) auf Rückmeldung zu drei eigenen Kästen geändert. Lokal und headless geprüft.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="22" t="inlineStr">
+        <is>
+          <t>REQ-63</t>
+        </is>
+      </c>
+      <c r="B43" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="C43" s="22" t="inlineStr">
+        <is>
+          <t>3.7.2</t>
+        </is>
+      </c>
+      <c r="D43" s="22" t="inlineStr">
+        <is>
+          <t>on the bottom it should be 3 columns of the boxes not one big on the left und two under each other on the right. then the left box whne clixking enlarge a separate window opes</t>
+        </is>
+      </c>
+      <c r="E43" s="22" t="inlineStr">
+        <is>
+          <t>Die B-Seite MUSS Wissenskarte, „Projects &amp; clusters“ und Graph Chat in drei Spalten nebeneinander zeigen. „Enlarge“ an der Wissenskarte MUSS ein eigenes Fenster öffnen.</t>
+        </is>
+      </c>
+      <c r="F43" s="22" t="inlineStr">
+        <is>
+          <t>Bei Desktop-Breite drei gleich hohe Spalten; „Enlarge“ öffnet ein Browserfenster nur mit der Wissenskarte; dort gewählte Cluster gelten für die Chats im Hauptfenster und umgekehrt; bei blockiertem Pop-up Vergrößerung über der Seite.</t>
+        </is>
+      </c>
+      <c r="G43" s="22" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="H43" s="22" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="I43" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="J43" s="22" t="inlineStr">
+        <is>
+          <t>Grid map|cluster|chat; map-window.js mit ?view=map und BroadcastChannel. Lokal und headless geprüft.</t>
         </is>
       </c>
     </row>
@@ -4979,7 +5063,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="130" customWidth="1" style="10" min="1" max="1"/>
@@ -5160,10 +5244,17 @@
         </is>
       </c>
     </row>
-    <row r="26">
+    <row r="26" s="11">
       <c r="A26" s="24" t="inlineStr">
         <is>
           <t>Release 3.7.1 (31.10.2026, Patch): REQ-62 (drei Kästen in einer Zeile auf der B-Seite).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="24" t="inlineStr">
+        <is>
+          <t>Release 3.7.2 (31.10.2026, Patch): REQ-63 (B-Seite in drei Spalten, Wissenskarte im eigenen Fenster).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ALITA v3.7.3 – larger question field; database bar over the map column (REQ-64, REQ-65)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiw6EWVWF8ScrYC2GD7
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -700,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F64"/>
+  <dimension ref="A1:F66"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -2726,7 +2726,7 @@
         </is>
       </c>
     </row>
-    <row r="64">
+    <row r="64" s="11">
       <c r="A64" s="22" t="inlineStr">
         <is>
           <t>REQ-63</t>
@@ -2755,6 +2755,70 @@
       <c r="F64" s="22" t="inlineStr">
         <is>
           <t>Grid map|cluster|chat; map-window.js.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" s="11">
+      <c r="A65" s="22" t="inlineStr">
+        <is>
+          <t>REQ-64</t>
+        </is>
+      </c>
+      <c r="B65" s="22" t="inlineStr">
+        <is>
+          <t>Größeres Eingabefeld in den Chats</t>
+        </is>
+      </c>
+      <c r="C65" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="D65" s="22" t="inlineStr">
+        <is>
+          <t>3.7.3</t>
+        </is>
+      </c>
+      <c r="E65" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 31.10.2026</t>
+        </is>
+      </c>
+      <c r="F65" s="22" t="inlineStr">
+        <is>
+          <t>4 Zeilen, wachsend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="22" t="inlineStr">
+        <is>
+          <t>REQ-65</t>
+        </is>
+      </c>
+      <c r="B66" s="22" t="inlineStr">
+        <is>
+          <t>Datenbankleiste so breit wie die Spalte der Wissenskarte</t>
+        </is>
+      </c>
+      <c r="C66" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="D66" s="22" t="inlineStr">
+        <is>
+          <t>3.7.3</t>
+        </is>
+      </c>
+      <c r="E66" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 31.10.2026</t>
+        </is>
+      </c>
+      <c r="F66" s="22" t="inlineStr">
+        <is>
+          <t>.bar-row-Grid.</t>
         </is>
       </c>
     </row>
@@ -2789,7 +2853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J43"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -4987,7 +5051,7 @@
         </is>
       </c>
     </row>
-    <row r="43">
+    <row r="43" s="11">
       <c r="A43" s="22" t="inlineStr">
         <is>
           <t>REQ-63</t>
@@ -5036,6 +5100,110 @@
       <c r="J43" s="22" t="inlineStr">
         <is>
           <t>Grid map|cluster|chat; map-window.js mit ?view=map und BroadcastChannel. Lokal und headless geprüft.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" s="11">
+      <c r="A44" s="22" t="inlineStr">
+        <is>
+          <t>REQ-64</t>
+        </is>
+      </c>
+      <c r="B44" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="C44" s="22" t="inlineStr">
+        <is>
+          <t>3.7.3</t>
+        </is>
+      </c>
+      <c r="D44" s="22" t="inlineStr">
+        <is>
+          <t>make the input area larger [Screenshot: Eingabefeld des Graph Chat]</t>
+        </is>
+      </c>
+      <c r="E44" s="22" t="inlineStr">
+        <is>
+          <t>Das Eingabefeld der Chats MUSS größer sein.</t>
+        </is>
+      </c>
+      <c r="F44" s="22" t="inlineStr">
+        <is>
+          <t>Leeres Feld mindestens vier Zeilen hoch; wächst mit dem Text; nach dem Senden wieder klein.</t>
+        </is>
+      </c>
+      <c r="G44" s="22" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="H44" s="22" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="I44" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="J44" s="22" t="inlineStr">
+        <is>
+          <t>min 104 px, max 280 px, vergrößerbar; beide Chats. Lokal geprüft.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="22" t="inlineStr">
+        <is>
+          <t>REQ-65</t>
+        </is>
+      </c>
+      <c r="B45" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="C45" s="22" t="inlineStr">
+        <is>
+          <t>3.7.3</t>
+        </is>
+      </c>
+      <c r="D45" s="22" t="inlineStr">
+        <is>
+          <t>extend the first box [Screenshot: Datenbankleiste, Pfeil nach rechts bis zum Rand der Wissenskarte]</t>
+        </is>
+      </c>
+      <c r="E45" s="22" t="inlineStr">
+        <is>
+          <t>Die Datenbankleiste (erster Kasten) MUSS auf der B-Seite bis zur Breite der Wissenskarten-Spalte reichen.</t>
+        </is>
+      </c>
+      <c r="F45" s="22" t="inlineStr">
+        <is>
+          <t>Rechte Kante der Datenbankleiste fluchtet mit der Wissenskarte; Fenster und Erklärung über den beiden anderen Spalten.</t>
+        </is>
+      </c>
+      <c r="G45" s="22" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="H45" s="22" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="I45" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="J45" s="22" t="inlineStr">
+        <is>
+          <t>.bar-row als Grid mit denselben Spalten wie die B-Seite. Lokal und headless geprüft.</t>
         </is>
       </c>
     </row>
@@ -5063,7 +5231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A27"/>
+  <dimension ref="A1:A28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="130" customWidth="1" style="10" min="1" max="1"/>
@@ -5251,10 +5419,17 @@
         </is>
       </c>
     </row>
-    <row r="27">
+    <row r="27" s="11">
       <c r="A27" s="24" t="inlineStr">
         <is>
           <t>Release 3.7.2 (31.10.2026, Patch): REQ-63 (B-Seite in drei Spalten, Wissenskarte im eigenen Fenster).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="24" t="inlineStr">
+        <is>
+          <t>Release 3.7.3 (31.10.2026, Patch): REQ-64 (größeres Eingabefeld), REQ-65 (Datenbankleiste über der Wissenskarte).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ALITA v3.8.0 – optional default OpenRouter key; an entered key wins (REQ-66)
- effective_key dependency behind X-OpenRouter-Key: own key, else
  OPENROUTER_API_KEY of the instance (reviewers only with
  SERVER_KEY_FOR_REVIEWERS=true); /api/health reports server_key
- Front end: key status "default key"
- .env.example / README / manual updated; tests 191 passed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiw6EWVWF8ScrYC2GD7
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -700,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F67"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -2790,7 +2790,7 @@
         </is>
       </c>
     </row>
-    <row r="66">
+    <row r="66" s="11">
       <c r="A66" s="22" t="inlineStr">
         <is>
           <t>REQ-65</t>
@@ -2819,6 +2819,38 @@
       <c r="F66" s="22" t="inlineStr">
         <is>
           <t>.bar-row-Grid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="22" t="inlineStr">
+        <is>
+          <t>REQ-66</t>
+        </is>
+      </c>
+      <c r="B67" s="22" t="inlineStr">
+        <is>
+          <t>Standard-OpenRouter-Key, eigener Key hat Vorrang</t>
+        </is>
+      </c>
+      <c r="C67" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="D67" s="22" t="inlineStr">
+        <is>
+          <t>3.8.0</t>
+        </is>
+      </c>
+      <c r="E67" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 31.10.2026</t>
+        </is>
+      </c>
+      <c r="F67" s="22" t="inlineStr">
+        <is>
+          <t>OPENROUTER_API_KEY in .env; effective_key.</t>
         </is>
       </c>
     </row>
@@ -2853,7 +2885,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -5155,7 +5187,7 @@
         </is>
       </c>
     </row>
-    <row r="45">
+    <row r="45" s="11">
       <c r="A45" s="22" t="inlineStr">
         <is>
           <t>REQ-65</t>
@@ -5204,6 +5236,58 @@
       <c r="J45" s="22" t="inlineStr">
         <is>
           <t>.bar-row als Grid mit denselben Spalten wie die B-Seite. Lokal und headless geprüft.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="22" t="inlineStr">
+        <is>
+          <t>REQ-66</t>
+        </is>
+      </c>
+      <c r="B46" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="C46" s="22" t="inlineStr">
+        <is>
+          <t>3.8.0</t>
+        </is>
+      </c>
+      <c r="D46" s="22" t="inlineStr">
+        <is>
+          <t>OpenRouter key is default set but can also be entered another one: [OPENROUTER_API_KEY=… – Key im Chat genannt, hier nicht protokolliert]</t>
+        </is>
+      </c>
+      <c r="E46" s="22" t="inlineStr">
+        <is>
+          <t>Die Instanz MUSS einen Standard-OpenRouter-Key haben können, der gilt, wenn im Interface kein eigener Key eingetragen ist; ein im Interface eingetragener Key MUSS Vorrang haben. Der Key DARF NICHT im Repository stehen.</t>
+        </is>
+      </c>
+      <c r="F46" s="22" t="inlineStr">
+        <is>
+          <t>Mit OPENROUTER_API_KEY in .env: Fragen ohne eingetragenen Key funktionieren, Status „default key“; mit eingetragenem Key wird dieser verwendet; ohne Standard-Key wie bisher 401.</t>
+        </is>
+      </c>
+      <c r="G46" s="22" t="inlineStr">
+        <is>
+          <t>Backend · Frontend · Sicherheit</t>
+        </is>
+      </c>
+      <c r="H46" s="22" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="I46" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="J46" s="22" t="inlineStr">
+        <is>
+          <t>effective_key-Dependency; anonyme Reviewer nur mit SERVER_KEY_FOR_REVIEWERS=true. Key selbst nur in .env (vom Nutzer einzutragen). Tests 3 neu.</t>
         </is>
       </c>
     </row>
@@ -5231,7 +5315,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A28"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="130" customWidth="1" style="10" min="1" max="1"/>
@@ -5426,10 +5510,17 @@
         </is>
       </c>
     </row>
-    <row r="28">
+    <row r="28" s="11">
       <c r="A28" s="24" t="inlineStr">
         <is>
           <t>Release 3.7.3 (31.10.2026, Patch): REQ-64 (größeres Eingabefeld), REQ-65 (Datenbankleiste über der Wissenskarte).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="24" t="inlineStr">
+        <is>
+          <t>Release 3.8.0 (31.10.2026, Minor): REQ-66 (optionaler Standard-Key der Instanz).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert "ALITA v3.8.0 – optional default OpenRouter key" (REQ-66 withdrawn)
Back to 3.7.3: every person enters their own OpenRouter key; a key in .env
is not used for chats. REQ-66 logged as withdrawn.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiw6EWVWF8ScrYC2GD7
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -2830,17 +2830,17 @@
       </c>
       <c r="B67" s="22" t="inlineStr">
         <is>
-          <t>Standard-OpenRouter-Key, eigener Key hat Vorrang</t>
+          <t>Standard-OpenRouter-Key</t>
         </is>
       </c>
       <c r="C67" s="22" t="inlineStr">
         <is>
-          <t>Erledigt</t>
+          <t>Offen</t>
         </is>
       </c>
       <c r="D67" s="22" t="inlineStr">
         <is>
-          <t>3.8.0</t>
+          <t>–</t>
         </is>
       </c>
       <c r="E67" s="22" t="inlineStr">
@@ -2850,7 +2850,7 @@
       </c>
       <c r="F67" s="22" t="inlineStr">
         <is>
-          <t>OPENROUTER_API_KEY in .env; effective_key.</t>
+          <t>Zurückgezogen (verworfen); 3.8.0 zurückgenommen.</t>
         </is>
       </c>
     </row>
@@ -5252,22 +5252,22 @@
       </c>
       <c r="C46" s="22" t="inlineStr">
         <is>
-          <t>3.8.0</t>
+          <t>–</t>
         </is>
       </c>
       <c r="D46" s="22" t="inlineStr">
         <is>
-          <t>OpenRouter key is default set but can also be entered another one: [OPENROUTER_API_KEY=… – Key im Chat genannt, hier nicht protokolliert]</t>
+          <t>OpenRouter key is default set but can also be entered another one: [Key im Chat genannt, hier nicht protokolliert] · später: „ok then reverese the last step“</t>
         </is>
       </c>
       <c r="E46" s="22" t="inlineStr">
         <is>
-          <t>Die Instanz MUSS einen Standard-OpenRouter-Key haben können, der gilt, wenn im Interface kein eigener Key eingetragen ist; ein im Interface eingetragener Key MUSS Vorrang haben. Der Key DARF NICHT im Repository stehen.</t>
+          <t>Die Instanz SOLL einen Standard-OpenRouter-Key haben können; ein im Interface eingetragener Key hat Vorrang.</t>
         </is>
       </c>
       <c r="F46" s="22" t="inlineStr">
         <is>
-          <t>Mit OPENROUTER_API_KEY in .env: Fragen ohne eingetragenen Key funktionieren, Status „default key“; mit eingetragenem Key wird dieser verwendet; ohne Standard-Key wie bisher 401.</t>
+          <t>–</t>
         </is>
       </c>
       <c r="G46" s="22" t="inlineStr">
@@ -5282,12 +5282,12 @@
       </c>
       <c r="I46" s="22" t="inlineStr">
         <is>
-          <t>Erledigt</t>
+          <t>Verworfen</t>
         </is>
       </c>
       <c r="J46" s="22" t="inlineStr">
         <is>
-          <t>effective_key-Dependency; anonyme Reviewer nur mit SERVER_KEY_FOR_REVIEWERS=true. Key selbst nur in .env (vom Nutzer einzutragen). Tests 3 neu.</t>
+          <t>Als 3.8.0 umgesetzt und auf Wunsch per Revert zurückgenommen; es bleibt dabei, dass jede Person ihren eigenen Key einträgt.</t>
         </is>
       </c>
     </row>
@@ -5315,7 +5315,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="130" customWidth="1" style="10" min="1" max="1"/>
@@ -5510,17 +5510,10 @@
         </is>
       </c>
     </row>
-    <row r="28" s="11">
+    <row r="28">
       <c r="A28" s="24" t="inlineStr">
         <is>
           <t>Release 3.7.3 (31.10.2026, Patch): REQ-64 (größeres Eingabefeld), REQ-65 (Datenbankleiste über der Wissenskarte).</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="24" t="inlineStr">
-        <is>
-          <t>Release 3.8.0 (31.10.2026, Minor): REQ-66 (optionaler Standard-Key der Instanz).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ALITA v3.9.0 – ask about what the knowledge map shows (REQ-67)
- cluster_query.py: clusters named in the question ("C8", "cluster 9")
  become the search space (across databases, project scope dropped);
  per-cluster retrieval; bridging passages = closest passage of the other
  cluster for the best passages of each (reference lists excluded)
- Prompt gets cluster profiles, the map relation and the passage pairs;
  graph path cluster -> document -> section (DEO/article) <-> section ->
  document -> cluster; answer footer lists the passage pairs
- Fixes: clusters always sent with the Graph Chat request; relation click
  clears a project scope; start-up race "DOCS is not defined"
- Tests 191 passed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiw6EWVWF8ScrYC2GD7
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -700,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F67"/>
+  <dimension ref="A1:F68"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -2822,7 +2822,7 @@
         </is>
       </c>
     </row>
-    <row r="67">
+    <row r="67" s="11">
       <c r="A67" s="22" t="inlineStr">
         <is>
           <t>REQ-66</t>
@@ -2851,6 +2851,38 @@
       <c r="F67" s="22" t="inlineStr">
         <is>
           <t>Zurückgezogen (verworfen); 3.8.0 zurückgenommen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="22" t="inlineStr">
+        <is>
+          <t>REQ-67</t>
+        </is>
+      </c>
+      <c r="B68" s="22" t="inlineStr">
+        <is>
+          <t>Fragen zu Zusammenhängen auf der Wissenskarte; Textstellen über die Ontologie</t>
+        </is>
+      </c>
+      <c r="C68" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="D68" s="22" t="inlineStr">
+        <is>
+          <t>3.9.0</t>
+        </is>
+      </c>
+      <c r="E68" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 31.10.2026</t>
+        </is>
+      </c>
+      <c r="F68" s="22" t="inlineStr">
+        <is>
+          <t>Cluster-Modus, Brücken-Stellen, Ontologie-Pfad.</t>
         </is>
       </c>
     </row>
@@ -2885,7 +2917,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J46"/>
+  <dimension ref="A1:J47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -5239,7 +5271,7 @@
         </is>
       </c>
     </row>
-    <row r="46">
+    <row r="46" s="11">
       <c r="A46" s="22" t="inlineStr">
         <is>
           <t>REQ-66</t>
@@ -5288,6 +5320,58 @@
       <c r="J46" s="22" t="inlineStr">
         <is>
           <t>Als 3.8.0 umgesetzt und auf Wunsch per Revert zurückgenommen; es bleibt dabei, dass jede Person ihren eigenen Key einträgt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="22" t="inlineStr">
+        <is>
+          <t>REQ-67</t>
+        </is>
+      </c>
+      <c r="B47" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="C47" s="22" t="inlineStr">
+        <is>
+          <t>3.9.0</t>
+        </is>
+      </c>
+      <c r="D47" s="22" t="inlineStr">
+        <is>
+          <t>Mehrwehrt entsteht wenn ich auch basierend auf dem was ich auf dem clusterbild sehe fragen stellen kann zu den zusammenhängen. also muss ja irghendwie über die onotolgie die text chunkjs angeteuer werden weisst du wie ich meine: [Screenshot: Graph Chat beantwortet „please describe the link between c8 and c9“ nur aus dem Weißbuch, Scope „project EU-AI-Act“]</t>
+        </is>
+      </c>
+      <c r="E47" s="22" t="inlineStr">
+        <is>
+          <t>Der Graph Chat MUSS Fragen zu den in der Wissenskarte sichtbaren Zusammenhängen beantworten können: in der Frage genannte Cluster MÜSSEN der Suchraum sein (auch über Datenbanken und trotz gewähltem Projekt), und der Weg zu den Textstellen MUSS über die Ontologie führen (Cluster → Dokument → Abschnitt mit DEO-Rolle/Rechtsbestandteil → Textstelle).</t>
+        </is>
+      </c>
+      <c r="F47" s="22" t="inlineStr">
+        <is>
+          <t>„describe the link between C8 and C9“ liefert Quellen aus beiden Clustern und Brücken-Stellen (ähnlichste Stellen über die Clustergrenze) mit Ähnlichkeit; der Graphpfad zeigt Cluster → Dokument → Abschnitt ↔ Abschnitt → Dokument → Cluster; die Antwort vergleicht beide Seiten.</t>
+        </is>
+      </c>
+      <c r="G47" s="22" t="inlineStr">
+        <is>
+          <t>Graph Chat · Backend · Ontologie</t>
+        </is>
+      </c>
+      <c r="H47" s="22" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="I47" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="J47" s="22" t="inlineStr">
+        <is>
+          <t>cluster_query.py (named_clusters, profiles, bridge_passages, bridge_path), Graph Chat Cluster-Modus, store.chunk_vectors. Live-Daten: Stellen aus C8 finden ihre Partner in C9 (z. B. 0,64). Tests 191 passed.</t>
         </is>
       </c>
     </row>
@@ -5315,7 +5399,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A28"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="130" customWidth="1" style="10" min="1" max="1"/>
@@ -5510,10 +5594,17 @@
         </is>
       </c>
     </row>
-    <row r="28">
+    <row r="28" s="11">
       <c r="A28" s="24" t="inlineStr">
         <is>
           <t>Release 3.7.3 (31.10.2026, Patch): REQ-64 (größeres Eingabefeld), REQ-65 (Datenbankleiste über der Wissenskarte).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="24" t="inlineStr">
+        <is>
+          <t>Release 3.9.0 (31.10.2026, Minor): REQ-67 (Fragen zu den Zusammenhängen auf der Wissenskarte, Brücken-Stellen).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ALITA v3.11.0 – papers per article, seen from the law (REQ-69)
- provisions.discussed_in: per article/annex/recital of a law version the
  papers that discuss it, in the numbering of that version (papers citing
  another version mapped over by the concordance); discusses keeps seq
- GET /api/legal/norms/{norm_id}/discussed?seq=
- Document details of a law version: "Discussed in papers" (only visible
  databases), click opens the paper, Ask fills the Graph Chat
- Tests 199 passed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiw6EWVWF8ScrYC2GD7
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -700,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F70"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -2915,6 +2915,38 @@
       <c r="F69" s="22" t="inlineStr">
         <is>
           <t>provisions.py: Verweise erkennen, Fassung bestimmen, auf geltende Nummern abbilden; DISCUSSES-Kanten, Graph Chat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="22" t="inlineStr">
+        <is>
+          <t>REQ-69</t>
+        </is>
+      </c>
+      <c r="B70" s="22" t="inlineStr">
+        <is>
+          <t>Je Artikel eines Gesetzes anzeigen, welche Paper ihn diskutieren</t>
+        </is>
+      </c>
+      <c r="C70" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="D70" s="22" t="inlineStr">
+        <is>
+          <t>3.11.0</t>
+        </is>
+      </c>
+      <c r="E70" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 31.10.2026</t>
+        </is>
+      </c>
+      <c r="F70" s="22" t="inlineStr">
+        <is>
+          <t>discussed_in, /api/legal/norms/{id}/discussed, Abschnitt „Discussed in papers“ mit Ask.</t>
         </is>
       </c>
     </row>
@@ -2949,7 +2981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J48"/>
+  <dimension ref="A1:J49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -5456,6 +5488,58 @@
       <c r="J48" s="22" t="inlineStr">
         <is>
           <t>provisions.py (find_refs, Resolver, link_document, rebuild, chat_scope, chat_passages); Payload discusses/provisions; Neo4j DISCUSSES/REFERS_TO; GET /api/provisions, POST /api/provisions/rebuild, CLI ingest provisions, automatisch nach jeder Ingestion. Offline mit den vier Fassungen des AI Act und beiden Wachter-Papern geprüft. Tests 198 passed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="22" t="inlineStr">
+        <is>
+          <t>REQ-69</t>
+        </is>
+      </c>
+      <c r="B49" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="C49" s="22" t="inlineStr">
+        <is>
+          <t>3.11.0</t>
+        </is>
+      </c>
+      <c r="D49" s="22" t="inlineStr">
+        <is>
+          <t>ja mach diesen schtizz [Antwort auf das Angebot: in der Gesetzesansicht je Artikel anzeigen, welche Paper ihn diskutieren]</t>
+        </is>
+      </c>
+      <c r="E49" s="22" t="inlineStr">
+        <is>
+          <t>Die Ansicht einer Gesetzesfassung MUSS je Artikel, Anhang und Erwägungsgrund die Paper zeigen, die ihn diskutieren – in der Nummerierung dieser Fassung, auch wenn ein Paper eine andere Fassung zitiert. Paper aus nicht sichtbaren Datenbanken DÜRFEN NICHT erscheinen. Von dort SOLL man das Paper öffnen und den Graph Chat fragen können.</t>
+        </is>
+      </c>
+      <c r="F49" s="22" t="inlineStr">
+        <is>
+          <t>Dokumentdetails „AI Act – Proposal“: Art. 33 „Notified bodies“ zeigt Laux et al. (4×, Art. 33(4)); in der konsolidierten Fassung erscheinen sie unter Art. 31 mit „cited as Art. 33 of the proposal“; Klick öffnet das Paper; „Ask“ schreibt „What do the papers say about Art. 31 of the AI Act (numbered 33 in the proposal)?“ in den Graph Chat.</t>
+        </is>
+      </c>
+      <c r="G49" s="22" t="inlineStr">
+        <is>
+          <t>Rechtstexte · Frontend · Backend</t>
+        </is>
+      </c>
+      <c r="H49" s="22" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="I49" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="J49" s="22" t="inlineStr">
+        <is>
+          <t>provisions.discussed_in (Rück-Konkordanz heutige Nummer → Nummer der Fassung), GET /api/legal/norms/{id}/discussed?seq=, legal.js loadLegalDiscussed. Offline: konsolidiert 72, Vorschlag 42 Bestimmungen mit Papern; Headless-Browser-Test. Tests 199 passed.</t>
         </is>
       </c>
     </row>
@@ -5483,7 +5567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:A31"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="130" customWidth="1" style="10" min="1" max="1"/>
@@ -5699,6 +5783,13 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="24" t="inlineStr">
+        <is>
+          <t>Release 3.11.0 (31.10.2026, Minor): REQ-69 (je Artikel die Paper, die ihn diskutieren, in der Nummerierung der Fassung).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
ALITA v3.12.0 – guided tour (REQ-70)
- Header button "Guided tour": eleven steps along the proposal's
  mechanisms (knowledge map, Compare, version history of a law, papers ->
  articles, law view, challenging questions, own projects with password;
  explore vs. exploit), spotlight on the explained element, example
  questions put into / asked in the Graph Chat
- Cluster numbers and example project from the current data; keys -> <-
  Esc; ?tour=1 starts it; hidden in the map window
- Checked in a headless browser on the demo data

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiw6EWVWF8ScrYC2GD7
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -700,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F70"/>
+  <dimension ref="A1:F71"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -2947,6 +2947,38 @@
       <c r="F70" s="22" t="inlineStr">
         <is>
           <t>discussed_in, /api/legal/norms/{id}/discussed, Abschnitt „Discussed in papers“ mit Ask.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="22" t="inlineStr">
+        <is>
+          <t>REQ-70</t>
+        </is>
+      </c>
+      <c r="B71" s="22" t="inlineStr">
+        <is>
+          <t>Knopf „Guided tour“, der durch ALITA führt</t>
+        </is>
+      </c>
+      <c r="C71" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="D71" s="22" t="inlineStr">
+        <is>
+          <t>3.12.0</t>
+        </is>
+      </c>
+      <c r="E71" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 31.10.2026</t>
+        </is>
+      </c>
+      <c r="F71" s="22" t="inlineStr">
+        <is>
+          <t>tour.js/tour.css: elf Schritte mit Hervorhebung und Beispielfragen für den Graph Chat.</t>
         </is>
       </c>
     </row>
@@ -2981,7 +3013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J49"/>
+  <dimension ref="A1:J50"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -5540,6 +5572,58 @@
       <c r="J49" s="22" t="inlineStr">
         <is>
           <t>provisions.discussed_in (Rück-Konkordanz heutige Nummer → Nummer der Fassung), GET /api/legal/norms/{id}/discussed?seq=, legal.js loadLegalDiscussed. Offline: konsolidiert 72, Vorschlag 42 Bestimmungen mit Papern; Headless-Browser-Test. Tests 199 passed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="22" t="inlineStr">
+        <is>
+          <t>REQ-70</t>
+        </is>
+      </c>
+      <c r="B50" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="C50" s="22" t="inlineStr">
+        <is>
+          <t>3.12.0</t>
+        </is>
+      </c>
+      <c r="D50" s="22" t="inlineStr">
+        <is>
+          <t>Can you add a button in alita like "showing tour" or better suitet name that when clicking on it it guides you</t>
+        </is>
+      </c>
+      <c r="E50" s="22" t="inlineStr">
+        <is>
+          <t>ALITA MUSS einen gut sichtbaren Knopf haben, der eine geführte Tour startet. Die Tour MUSS Schritt für Schritt die wichtigsten Teile zeigen (entlang der Mechanismen aus dem Forschungsantrag: Erinnerung auffrischen vertikal/horizontal, Nachvollziehbarkeit, Schemata aktualisieren) und SOLL Beispielfragen direkt in den Graph Chat übernehmen können. Sie MUSS ohne Passwort mit den öffentlichen Datenbanken funktionieren.</t>
+        </is>
+      </c>
+      <c r="F50" s="22" t="inlineStr">
+        <is>
+          <t>Klick auf „▶ Guided tour“ öffnet Schritt 1; Weiter/Zurück/Schließen und Tasten → ← Esc funktionieren; jeder Schritt wechselt auf die richtige Seite und hebt die erklärte Stelle hervor; „Put into Graph Chat“ setzt die Beispielfrage ins Eingabefeld, „Ask now“ sendet sie; keine Fehler in der Konsole.</t>
+        </is>
+      </c>
+      <c r="G50" s="22" t="inlineStr">
+        <is>
+          <t>Frontend · Onboarding</t>
+        </is>
+      </c>
+      <c r="H50" s="22" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="I50" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="J50" s="22" t="inlineStr">
+        <is>
+          <t>frontend/js/tour.js, css/tour.css, Knopf #tourBtn; Cluster-Nummern und Beispielprojekt aus den aktuellen Daten; ?tour=1. Headless-Browser-Test auf den Demodaten: 11 Schritte, alle Ziele gefunden, Fenster immer im Bild, keine Fehler.</t>
         </is>
       </c>
     </row>
@@ -5567,7 +5651,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A31"/>
+  <dimension ref="A1:A32"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="130" customWidth="1" style="10" min="1" max="1"/>
@@ -5790,6 +5874,13 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="24" t="inlineStr">
+        <is>
+          <t>Release 3.12.0 (31.10.2026, Minor): REQ-70 (Guided tour).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Add MIT licence (REQ-72); log REQ-71 (update the repository)
- LICENSE (MIT, Copyright 2026 ProDigi-Repo – ALITA contributors)
- README section "Lizenz": covers code and documentation; documents
  loaded into ALITA keep their own licences
- CHANGELOG [Unreleased], requirements status and log

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiw6EWVWF8ScrYC2GD7
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -700,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:F73"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -2979,6 +2979,70 @@
       <c r="F71" s="22" t="inlineStr">
         <is>
           <t>tour.js/tour.css: elf Schritte mit Hervorhebung und Beispielfragen für den Graph Chat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="22" t="inlineStr">
+        <is>
+          <t>REQ-71</t>
+        </is>
+      </c>
+      <c r="B72" s="22" t="inlineStr">
+        <is>
+          <t>GitHub-Repository aktualisieren (alle Releases nach main)</t>
+        </is>
+      </c>
+      <c r="C72" s="22" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
+        </is>
+      </c>
+      <c r="D72" s="22" t="inlineStr">
+        <is>
+          <t>3.6.2 – 3.12.0</t>
+        </is>
+      </c>
+      <c r="E72" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 31.10.2026</t>
+        </is>
+      </c>
+      <c r="F72" s="22" t="inlineStr">
+        <is>
+          <t>PR #9 und #10 grün und mergebar; Merge durch Maintainer (#9 zuerst).</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="22" t="inlineStr">
+        <is>
+          <t>REQ-72</t>
+        </is>
+      </c>
+      <c r="B73" s="22" t="inlineStr">
+        <is>
+          <t>MIT-Lizenz ergänzen</t>
+        </is>
+      </c>
+      <c r="C73" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="D73" s="22" t="inlineStr">
+        <is>
+          <t>Unreleased</t>
+        </is>
+      </c>
+      <c r="E73" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 31.10.2026</t>
+        </is>
+      </c>
+      <c r="F73" s="22" t="inlineStr">
+        <is>
+          <t>LICENSE (MIT), Abschnitt „Lizenz“ im README; im PR #10.</t>
         </is>
       </c>
     </row>
@@ -3013,7 +3077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J50"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -5624,6 +5688,110 @@
       <c r="J50" s="22" t="inlineStr">
         <is>
           <t>frontend/js/tour.js, css/tour.css, Knopf #tourBtn; Cluster-Nummern und Beispielprojekt aus den aktuellen Daten; ?tour=1. Headless-Browser-Test auf den Demodaten: 11 Schritte, alle Ziele gefunden, Fenster immer im Bild, keine Fehler.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="22" t="inlineStr">
+        <is>
+          <t>REQ-71</t>
+        </is>
+      </c>
+      <c r="B51" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="C51" s="22" t="inlineStr">
+        <is>
+          <t>3.12.0</t>
+        </is>
+      </c>
+      <c r="D51" s="22" t="inlineStr">
+        <is>
+          <t>update the github reposity: https://github.com/ProDigi-Repo/ALITA</t>
+        </is>
+      </c>
+      <c r="E51" s="22" t="inlineStr">
+        <is>
+          <t>Der Stand 3.6.2 – 3.12.0 MUSS im GitHub-Repository auf main ankommen; PR #9 MUSS vor PR #10 gemergt werden.</t>
+        </is>
+      </c>
+      <c r="F51" s="22" t="inlineStr">
+        <is>
+          <t>main enthält VERSION 3.12.0; CI auf main grün.</t>
+        </is>
+      </c>
+      <c r="G51" s="22" t="inlineStr">
+        <is>
+          <t>Repository · Release</t>
+        </is>
+      </c>
+      <c r="H51" s="22" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="I51" s="22" t="inlineStr">
+        <is>
+          <t>In Arbeit</t>
+        </is>
+      </c>
+      <c r="J51" s="22" t="inlineStr">
+        <is>
+          <t>Alles auf die PR-Branches gepusht, PR-Beschreibungen aktuell, CI grün. Der Merge nach main ohne Review war für Claude gesperrt – Merge durch einen Maintainer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="22" t="inlineStr">
+        <is>
+          <t>REQ-72</t>
+        </is>
+      </c>
+      <c r="B52" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="C52" s="22" t="inlineStr">
+        <is>
+          <t>Unreleased</t>
+        </is>
+      </c>
+      <c r="D52" s="22" t="inlineStr">
+        <is>
+          <t>add a mIT licencse</t>
+        </is>
+      </c>
+      <c r="E52" s="22" t="inlineStr">
+        <is>
+          <t>Das Repository MUSS eine MIT-Lizenzdatei enthalten; das README SOLL auf sie verweisen und klarstellen, dass eingelesene Dokumente ihre eigenen Lizenzen behalten.</t>
+        </is>
+      </c>
+      <c r="F52" s="22" t="inlineStr">
+        <is>
+          <t>LICENSE mit dem MIT-Text im Wurzelverzeichnis; GitHub zeigt „MIT license“; README-Abschnitt „Lizenz“.</t>
+        </is>
+      </c>
+      <c r="G52" s="22" t="inlineStr">
+        <is>
+          <t>Repository · Recht</t>
+        </is>
+      </c>
+      <c r="H52" s="22" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="I52" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="J52" s="22" t="inlineStr">
+        <is>
+          <t>LICENSE (Copyright 2026 ProDigi-Repo – ALITA contributors), README-Abschnitt, CHANGELOG [Unreleased]. Im PR #10, landet mit dem Merge auf main.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Document the copyright status of the EU AI Act database (REQ-73)
- docs/compliance/05: legal acts are official works without copyright
  (e.g. § 5(1) UrhG; EUR-Lex reuse under Decision 2011/833/EU, consolidated
  texts CC BY 4.0); Commission documents reusable with attribution;
  NIST SP 800-18r2 a US government work (17 U.S.C. § 105); purchased
  standards and the Wachter papers excluded
- README "Lizenz", CHANGELOG [Unreleased], requirements status and log

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiw6EWVWF8ScrYC2GD7
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -700,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F73"/>
+  <dimension ref="A1:F74"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -3043,6 +3043,38 @@
       <c r="F73" s="22" t="inlineStr">
         <is>
           <t>LICENSE (MIT), Abschnitt „Lizenz“ im README; im PR #10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="22" t="inlineStr">
+        <is>
+          <t>REQ-73</t>
+        </is>
+      </c>
+      <c r="B74" s="22" t="inlineStr">
+        <is>
+          <t>Beschreiben, dass die Daten der Datenbank EU AI Act Rechtstexte und daher nicht urheberrechtlich geschützt sind</t>
+        </is>
+      </c>
+      <c r="C74" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="D74" s="22" t="inlineStr">
+        <is>
+          <t>Unreleased</t>
+        </is>
+      </c>
+      <c r="E74" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 31.10.2026</t>
+        </is>
+      </c>
+      <c r="F74" s="22" t="inlineStr">
+        <is>
+          <t>Abschnitt in docs/compliance/05, README „Lizenz“, research/EUAIA/README.md.</t>
         </is>
       </c>
     </row>
@@ -3077,7 +3109,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J52"/>
+  <dimension ref="A1:J53"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -5792,6 +5824,58 @@
       <c r="J52" s="22" t="inlineStr">
         <is>
           <t>LICENSE (Copyright 2026 ProDigi-Repo – ALITA contributors), README-Abschnitt, CHANGELOG [Unreleased]. Im PR #10, landet mit dem Merge auf main.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="22" t="inlineStr">
+        <is>
+          <t>REQ-73</t>
+        </is>
+      </c>
+      <c r="B53" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="C53" s="22" t="inlineStr">
+        <is>
+          <t>Unreleased</t>
+        </is>
+      </c>
+      <c r="D53" s="22" t="inlineStr">
+        <is>
+          <t>describe that the data in eu ai act database is legal text and thus not protected by copyright</t>
+        </is>
+      </c>
+      <c r="E53" s="22" t="inlineStr">
+        <is>
+          <t>Die Dokumentation MUSS beschreiben, dass die Datenbank EU AI Act aus Rechtstexten und amtlichen Dokumenten besteht und die Rechtstexte nicht urheberrechtlich geschützt sind; sie SOLL je Dokumentgruppe die Grundlage nennen und Abweichungen (amtliche Dokumente mit Quellenangabe, gekaufte Normen, Paper der Datenbank Wachter) klar abgrenzen.</t>
+        </is>
+      </c>
+      <c r="F53" s="22" t="inlineStr">
+        <is>
+          <t>Abschnitt „Copyright status of the database EU AI Act“ in docs/compliance/05 mit Tabelle je Dokumentgruppe; Hinweis im README; research/EUAIA/README.md mit gleichem Inhalt.</t>
+        </is>
+      </c>
+      <c r="G53" s="22" t="inlineStr">
+        <is>
+          <t>Dokumentation · Recht</t>
+        </is>
+      </c>
+      <c r="H53" s="22" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="I53" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="J53" s="22" t="inlineStr">
+        <is>
+          <t>Grundlagen geprüft: § 5 Abs. 1 UrhG; EUR-Lex-Hinweis (Weiterverwendung nach Beschluss 2011/833/EU, konsolidierte Texte CC BY 4.0); NIST 17 U.S.C. § 105. Keine Rechtsberatung.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Requirements: REQ-71 done (PR #9 and #10 merged)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiw6EWVWF8ScrYC2GD7
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -2995,7 +2995,7 @@
       </c>
       <c r="C72" s="22" t="inlineStr">
         <is>
-          <t>In Arbeit</t>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="D72" s="22" t="inlineStr">
@@ -3010,7 +3010,7 @@
       </c>
       <c r="F72" s="22" t="inlineStr">
         <is>
-          <t>PR #9 und #10 grün und mergebar; Merge durch Maintainer (#9 zuerst).</t>
+          <t>PR #9 und #10 gemergt; main auf 3.12.0.</t>
         </is>
       </c>
     </row>
@@ -5766,12 +5766,12 @@
       </c>
       <c r="I51" s="22" t="inlineStr">
         <is>
-          <t>In Arbeit</t>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="J51" s="22" t="inlineStr">
         <is>
-          <t>Alles auf die PR-Branches gepusht, PR-Beschreibungen aktuell, CI grün. Der Merge nach main ohne Review war für Claude gesperrt – Merge durch einen Maintainer.</t>
+          <t>Alles auf die PR-Branches gepusht; PR #9 und #10 am 31.10.2026 von der Nutzerin gemergt; main auf 3.12.0 mit MIT-Lizenz.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ALITA v3.13.0 – refactoring done (REQ-74, REQ-61 stages 1–5)
- version 3.13.0; CHANGELOG: Unreleased entries (licence, copyright, deployment, security) move into 3.13.0
- refactoring plan marked done, with 'How to add things now' and how behaviour was checked
- README code map, ingestion CLI, version table; ingestion doc points to app/ingestion/
- requirements log: REQ-74 logged, REQ-61 done, REQ-72/73 released in 3.13.0

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiutQb1DRNGi5QGNWTT
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -700,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F74"/>
+  <dimension ref="A1:F75"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -2675,12 +2675,12 @@
       </c>
       <c r="C62" s="22" t="inlineStr">
         <is>
-          <t>In Arbeit</t>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="D62" s="22" t="inlineStr">
         <is>
-          <t>3.7.0 –</t>
+          <t>3.7.0 – 3.13.0</t>
         </is>
       </c>
       <c r="E62" s="22" t="inlineStr">
@@ -2690,7 +2690,7 @@
       </c>
       <c r="F62" s="22" t="inlineStr">
         <is>
-          <t>Stufe 0 erledigt; Plan in docs/technical/architecture.</t>
+          <t>Stufe 0 in 3.7.0; Stufen 1–5 in 3.13.0 (REQ-74): Router je Fachgebiet, gemeinsamer Scope für A und B, Ingestion-Paket, Datenbank-Registry, Frontend-Ereignisse (state.js), clusters.js aufgeteilt.</t>
         </is>
       </c>
     </row>
@@ -3032,7 +3032,7 @@
       </c>
       <c r="D73" s="22" t="inlineStr">
         <is>
-          <t>Unreleased</t>
+          <t>3.13.0</t>
         </is>
       </c>
       <c r="E73" s="22" t="inlineStr">
@@ -3046,7 +3046,7 @@
         </is>
       </c>
     </row>
-    <row r="74">
+    <row r="74" s="11">
       <c r="A74" s="22" t="inlineStr">
         <is>
           <t>REQ-73</t>
@@ -3064,7 +3064,7 @@
       </c>
       <c r="D74" s="22" t="inlineStr">
         <is>
-          <t>Unreleased</t>
+          <t>3.13.0</t>
         </is>
       </c>
       <c r="E74" s="22" t="inlineStr">
@@ -3075,6 +3075,38 @@
       <c r="F74" s="22" t="inlineStr">
         <is>
           <t>Abschnitt in docs/compliance/05, README „Lizenz“, research/EUAIA/README.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="22" t="inlineStr">
+        <is>
+          <t>REQ-74</t>
+        </is>
+      </c>
+      <c r="B75" s="22" t="inlineStr">
+        <is>
+          <t>Großes Refactoring als Grundlage für neue Funktionen (ohne sichtbare Änderung)</t>
+        </is>
+      </c>
+      <c r="C75" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="D75" s="22" t="inlineStr">
+        <is>
+          <t>3.13.0</t>
+        </is>
+      </c>
+      <c r="E75" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 01.11.2026</t>
+        </is>
+      </c>
+      <c r="F75" s="22" t="inlineStr">
+        <is>
+          <t>Siehe REQ-61, Stufen 1–5; Verhalten gegen main geprüft (API, UI-Zustände, Tour, Kartenfenster).</t>
         </is>
       </c>
     </row>
@@ -3109,7 +3141,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J53"/>
+  <dimension ref="A1:J54"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -5788,7 +5820,7 @@
       </c>
       <c r="C52" s="22" t="inlineStr">
         <is>
-          <t>Unreleased</t>
+          <t>3.13.0</t>
         </is>
       </c>
       <c r="D52" s="22" t="inlineStr">
@@ -5827,7 +5859,7 @@
         </is>
       </c>
     </row>
-    <row r="53">
+    <row r="53" s="11">
       <c r="A53" s="22" t="inlineStr">
         <is>
           <t>REQ-73</t>
@@ -5840,7 +5872,7 @@
       </c>
       <c r="C53" s="22" t="inlineStr">
         <is>
-          <t>Unreleased</t>
+          <t>3.13.0</t>
         </is>
       </c>
       <c r="D53" s="22" t="inlineStr">
@@ -5876,6 +5908,58 @@
       <c r="J53" s="22" t="inlineStr">
         <is>
           <t>Grundlagen geprüft: § 5 Abs. 1 UrhG; EUR-Lex-Hinweis (Weiterverwendung nach Beschluss 2011/833/EU, konsolidierte Texte CC BY 4.0); NIST 17 U.S.C. § 105. Keine Rechtsberatung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="22" t="inlineStr">
+        <is>
+          <t>REQ-74</t>
+        </is>
+      </c>
+      <c r="B54" s="22" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="C54" s="22" t="inlineStr">
+        <is>
+          <t>3.13.0</t>
+        </is>
+      </c>
+      <c r="D54" s="22" t="inlineStr">
+        <is>
+          <t>Now it is time to make a big fat clean refactoring of the code such that we can continue with new functionalities. Please do so</t>
+        </is>
+      </c>
+      <c r="E54" s="22" t="inlineStr">
+        <is>
+          <t>Der Code MUSS so umgebaut werden, dass neue Funktionen an einer Stelle ergänzt werden können: Backend-Routen nach Fachgebiet getrennt, eine gemeinsame Such-Reichweite (Scope) für Document Chat und Graph Chat, eine aufgeteilte Ingestion-Pipeline, eine Datenbank-Registry als einzige Quelle und Änderungs-Ereignisse im Frontend. Oberfläche und API DÜRFEN sich dabei NICHT ändern (gewollte Ausnahme laut Plan, Stufe 2: der Document Chat sucht bei mehreren Datenbanken je Datenbank, wie der Graph Chat).</t>
+        </is>
+      </c>
+      <c r="F54" s="22" t="inlineStr">
+        <is>
+          <t>Gleiche Routen und Methoden wie auf main; alle GET-Antworten auf denselben Daten gleich (außer den neuen Registry-Feldern); pytest, ruff, node --check und build_frontend ohne Diff grün; gleiche UI-Zustände nach derselben Klickfolge (Passwort, Datenbanken, Cluster, Compare, Kartenfenster, Guided Tour).</t>
+        </is>
+      </c>
+      <c r="G54" s="22" t="inlineStr">
+        <is>
+          <t>Architektur · Backend · Frontend</t>
+        </is>
+      </c>
+      <c r="H54" s="22" t="inlineStr">
+        <is>
+          <t>Hoch</t>
+        </is>
+      </c>
+      <c r="I54" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="J54" s="22" t="inlineStr">
+        <is>
+          <t>Stufen 1–5 aus docs/technical/architecture/01-refactoring-plan.md (REQ-61) umgesetzt: app/routes/, app/retrieval.py (Scope), app/ingestion/, app/registry.py + css/databases.css (generiert), js/state.js; clusters.js in fünf Dateien. Zugriffstests prüfen wieder jede Route (route_table, neuere FastAPI listet eingebundene Router nicht mehr in app.routes). Nebenbei behoben: Parameterzeile von A folgt der Cluster-Auswahl, Parameterzeile von B zeigt ein angeklicktes Projekt sofort. 205 Tests (199 vorher + 6 neue).</t>
         </is>
       </c>
     </row>
@@ -5903,7 +5987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A32"/>
+  <dimension ref="A1:A33"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="130" customWidth="1" style="10" min="1" max="1"/>
@@ -6126,10 +6210,17 @@
         </is>
       </c>
     </row>
-    <row r="32">
+    <row r="32" s="11">
       <c r="A32" s="24" t="inlineStr">
         <is>
           <t>Release 3.12.0 (31.10.2026, Minor): REQ-70 (Guided tour).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="24" t="inlineStr">
+        <is>
+          <t>Release 3.13.0 (01.11.2026, Minor): REQ-74 (Refactoring, REQ-61 Stufen 1–5); enthält auch REQ-72 (MIT-Lizenz) und REQ-73 (Urheberrecht EU AI Act).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove the 'Window to the outside' row (REQ-75); A/B Interaction Interface only with the password (REQ-76)
- B page: the row with 'Window to the outside' and the B explainer is gone, with its pop-up window,
  outside.js, outside.css and desert.css; the database bar spans the full width
- LOCKED_PAGES gets 'chat': without the password only B and Documents are shown
- user manual, CHANGELOG 3.13.0, requirements log and status updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiutQb1DRNGi5QGNWTT
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -700,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F75"/>
+  <dimension ref="A1:F77"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -3107,6 +3107,70 @@
       <c r="F75" s="22" t="inlineStr">
         <is>
           <t>Siehe REQ-61, Stufen 1–5; Verhalten gegen main geprüft (API, UI-Zustände, Tour, Kartenfenster).</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="22" t="inlineStr">
+        <is>
+          <t>REQ-75</t>
+        </is>
+      </c>
+      <c r="B76" s="22" t="inlineStr">
+        <is>
+          <t>Zeile „Window to the outside“ + B-Erklärung entfernen</t>
+        </is>
+      </c>
+      <c r="C76" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="D76" s="22" t="inlineStr">
+        <is>
+          <t>3.13.0</t>
+        </is>
+      </c>
+      <c r="E76" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 01.11.2026</t>
+        </is>
+      </c>
+      <c r="F76" s="22" t="inlineStr">
+        <is>
+          <t>Zeile und Pop-up-Fenster samt outside.js/outside.css/desert.css entfernt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="22" t="inlineStr">
+        <is>
+          <t>REQ-76</t>
+        </is>
+      </c>
+      <c r="B77" s="22" t="inlineStr">
+        <is>
+          <t>A/B Interaction Interface nur mit Passwort</t>
+        </is>
+      </c>
+      <c r="C77" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="D77" s="22" t="inlineStr">
+        <is>
+          <t>3.13.0</t>
+        </is>
+      </c>
+      <c r="E77" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 01.11.2026</t>
+        </is>
+      </c>
+      <c r="F77" s="22" t="inlineStr">
+        <is>
+          <t>LOCKED_PAGES um 'chat' ergänzt.</t>
         </is>
       </c>
     </row>
@@ -3141,7 +3205,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:J56"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -5960,6 +6024,110 @@
       <c r="J54" s="22" t="inlineStr">
         <is>
           <t>Stufen 1–5 aus docs/technical/architecture/01-refactoring-plan.md (REQ-61) umgesetzt: app/routes/, app/retrieval.py (Scope), app/ingestion/, app/registry.py + css/databases.css (generiert), js/state.js; clusters.js in fünf Dateien. Zugriffstests prüfen wieder jede Route (route_table, neuere FastAPI listet eingebundene Router nicht mehr in app.routes). Nebenbei behoben: Parameterzeile von A folgt der Cluster-Auswahl, Parameterzeile von B zeigt ein angeklicktes Projekt sofort. 205 Tests (199 vorher + 6 neue).</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="22" t="inlineStr">
+        <is>
+          <t>REQ-75</t>
+        </is>
+      </c>
+      <c r="B55" s="22" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="C55" s="22" t="inlineStr">
+        <is>
+          <t>3.13.0</t>
+        </is>
+      </c>
+      <c r="D55" s="22" t="inlineStr">
+        <is>
+          <t>remove this: [Screenshot: Zeile „Window to the outside“ + B-Erklärung „B searches the knowledge graph …“]</t>
+        </is>
+      </c>
+      <c r="E55" s="22" t="inlineStr">
+        <is>
+          <t>Die Zeile unter der Datenbankleiste der B-Seite (Kachel „Window to the outside“ und B-Erklärung) MUSS entfernt werden.</t>
+        </is>
+      </c>
+      <c r="F55" s="22" t="inlineStr">
+        <is>
+          <t>Kein #bTop/#bOutside im DOM; Datenbankleiste über die volle Breite; keine JS-Fehler; Guided Tour läuft durch.</t>
+        </is>
+      </c>
+      <c r="G55" s="22" t="inlineStr">
+        <is>
+          <t>Frontend · B-Seite</t>
+        </is>
+      </c>
+      <c r="H55" s="22" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="I55" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="J55" s="22" t="inlineStr">
+        <is>
+          <t>Zeile, Pop-up-Fenster, outside.js, outside.css, desert.css entfernt; Hinweis in info-alita.js und Regeln in tiles.css entfernt. REQ-20 (externe Prüfung) bleibt geplant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="22" t="inlineStr">
+        <is>
+          <t>REQ-76</t>
+        </is>
+      </c>
+      <c r="B56" s="22" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="C56" s="22" t="inlineStr">
+        <is>
+          <t>3.13.0</t>
+        </is>
+      </c>
+      <c r="D56" s="22" t="inlineStr">
+        <is>
+          <t>These are only visible when password is entered [Screenshot: Tabs A/B Interaction Interface, Release Notes, ISO 42001/EUAIACT Docs, Technical Documentation]</t>
+        </is>
+      </c>
+      <c r="E56" s="22" t="inlineStr">
+        <is>
+          <t>Der Tab „A/B Interaction Interface“ MUSS wie Release Notes, ISO 42001/EUAIACT Docs und Technical Documentation nur nach Eingabe des Passworts sichtbar sein.</t>
+        </is>
+      </c>
+      <c r="F56" s="22" t="inlineStr">
+        <is>
+          <t>Ohne Passwort nur „B Interaction Interface“ und „Documents“; #chat öffnet dann B; Sperren auf A/B wechselt zu B; mit Passwort alle sechs Tabs.</t>
+        </is>
+      </c>
+      <c r="G56" s="22" t="inlineStr">
+        <is>
+          <t>Frontend · Zugang</t>
+        </is>
+      </c>
+      <c r="H56" s="22" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="I56" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="J56" s="22" t="inlineStr">
+        <is>
+          <t>LOCKED_PAGES um 'chat' ergänzt (databases.js); im Browser geprüft (gesperrt, #chat, entsperren, wieder sperren).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Admin account gengar that sees all databases (REQ-78)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuMoiutQb1DRNGi5QGNWTT
</commit_message>
<xml_diff>
--- a/docs/requirements-log.xlsx
+++ b/docs/requirements-log.xlsx
@@ -700,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F78"/>
+  <dimension ref="A1:F79"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -3203,6 +3203,38 @@
       <c r="F78" s="22" t="inlineStr">
         <is>
           <t>Serverseitig durchgesetzt (visibility.py); Konten nur als Hashes außerhalb des Repositorys.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="22" t="inlineStr">
+        <is>
+          <t>REQ-78</t>
+        </is>
+      </c>
+      <c r="B79" s="22" t="inlineStr">
+        <is>
+          <t>Admin-Konto gengar, sieht alle Datenbanken</t>
+        </is>
+      </c>
+      <c r="C79" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="D79" s="22" t="inlineStr">
+        <is>
+          <t>3.13.0</t>
+        </is>
+      </c>
+      <c r="E79" s="22" t="inlineStr">
+        <is>
+          <t>Sitzung 01.11.2026</t>
+        </is>
+      </c>
+      <c r="F79" s="22" t="inlineStr">
+        <is>
+          <t>Ersetzt das Konto „admin“.</t>
         </is>
       </c>
     </row>
@@ -3237,7 +3269,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J57"/>
+  <dimension ref="A1:J58"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="10" min="1" max="1"/>
@@ -6212,6 +6244,58 @@
       <c r="J57" s="22" t="inlineStr">
         <is>
           <t>accounts.py (scrypt-Hashes, signiertes Session-Cookie, CLI import/set/remove/list), visibility.py (erlaubte Datenbanken je Anfrage, angewandt beim Lesen: Qdrant, Rechtsmodelle, Neo4j-Treffer), Routen /api/login, /api/logout, /api/accounts; Frontend #dbUser. 23 Konten + „All databases“ (bisheriges gemeinsames Passwort) in .secrets/accounts/accounts.json auf dem lokalen Rechner (gitignored); Datenbank-IDs = Benutzername in Großbuchstaben. Tests test_accounts.py (8) und Browserprüfung. Passwörter aus dem Screenshot abgetippt – bei Abweichungen mit `python -m app.accounts import` aus der Originaltabelle neu einlesen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="22" t="inlineStr">
+        <is>
+          <t>REQ-78</t>
+        </is>
+      </c>
+      <c r="B58" s="22" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="C58" s="22" t="inlineStr">
+        <is>
+          <t>3.13.0</t>
+        </is>
+      </c>
+      <c r="D58" s="22" t="inlineStr">
+        <is>
+          <t>I also need an admin who can see all. name should be gengar and password should be password</t>
+        </is>
+      </c>
+      <c r="E58" s="22" t="inlineStr">
+        <is>
+          <t>Es MUSS ein Konto „gengar“ geben, das alle Datenbanken sieht (Passwort wie vom Anforderer festgelegt).</t>
+        </is>
+      </c>
+      <c r="F58" s="22" t="inlineStr">
+        <is>
+          <t>Login als gengar zeigt alle Datenbanken und alle Tabs; im Dropdown steht gengar an erster Stelle.</t>
+        </is>
+      </c>
+      <c r="G58" s="22" t="inlineStr">
+        <is>
+          <t>Zugang · Konten</t>
+        </is>
+      </c>
+      <c r="H58" s="22" t="inlineStr">
+        <is>
+          <t>Mittel</t>
+        </is>
+      </c>
+      <c r="I58" s="22" t="inlineStr">
+        <is>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="J58" s="22" t="inlineStr">
+        <is>
+          <t>Konto gengar (database "*") in .secrets/accounts/accounts.json; das bisherige Konto „admin“ mit demselben Passwort entfernt. Passwort ist schwach – Hinweis an den Anforderer.</t>
         </is>
       </c>
     </row>

</xml_diff>